<commit_message>
LCSC and DigiKey  BOMs reviewed  and updated.
</commit_message>
<xml_diff>
--- a/Hardware-Designing/Deliverables/BOM/Digikey BOM.xlsx
+++ b/Hardware-Designing/Deliverables/BOM/Digikey BOM.xlsx
@@ -1,25 +1,35 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="5" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="24430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Github\ShockSensor-George\Hardware-Designing\Deliverables\BOM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark\ShockSensor-George\Hardware-Designing\Deliverables\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3EA5DE71-C923-4243-ADE7-8D9F39A7B8AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12495"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="282" uniqueCount="163">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="283" uniqueCount="170">
   <si>
     <t>Bill of Material (BOM) for  George (Rack Monitor)</t>
   </si>
@@ -528,17 +538,38 @@
   <si>
     <t xml:space="preserve">LED BLUE CLEAR 3MM T/H
 </t>
+  </si>
+  <si>
+    <t>Local supplier</t>
+  </si>
+  <si>
+    <t>will be arrange from custom supplier</t>
+  </si>
+  <si>
+    <t>Mouser</t>
+  </si>
+  <si>
+    <t>-------</t>
+  </si>
+  <si>
+    <t>--------</t>
+  </si>
+  <si>
+    <t>----------</t>
+  </si>
+  <si>
+    <t>-----------</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00000"/>
     <numFmt numFmtId="165" formatCode="_-[$$-409]* #,##0.00_ ;_-[$$-409]* \-#,##0.00\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
   </numFmts>
-  <fonts count="15">
+  <fonts count="18">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -614,13 +645,6 @@
     </font>
     <font>
       <sz val="10"/>
-      <color rgb="FFFF0000"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="10"/>
       <name val="Calibri"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -646,8 +670,40 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <strike/>
+      <sz val="10"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <strike/>
+      <u/>
+      <sz val="10"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <strike/>
+      <sz val="12"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -666,6 +722,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="32">
     <border>
@@ -1071,12 +1133,12 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="top"/>
       <protection locked="0"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="112">
+  <cellXfs count="127">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1096,9 +1158,6 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1181,9 +1240,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="3" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="165" fontId="9" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1"/>
@@ -1212,18 +1268,9 @@
     <xf numFmtId="164" fontId="5" fillId="3" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="165" fontId="10" fillId="3" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="11" fillId="3" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="165" fontId="10" fillId="3" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1239,9 +1286,6 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="14" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1266,12 +1310,6 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1299,24 +1337,6 @@
     <xf numFmtId="164" fontId="5" fillId="3" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1333,12 +1353,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="10" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1384,20 +1398,113 @@
     <xf numFmtId="164" fontId="5" fillId="3" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="16" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="28" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="12" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="16" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="28" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="12" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="6" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="7" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="18" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="4" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="4" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="13" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="9" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="10" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="4" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="12" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="13" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="4" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="4" borderId="10" xfId="1" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="13" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="4" borderId="13" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="4" borderId="10" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="17" fillId="4" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1674,7 +1781,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:Q35"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
@@ -1689,40 +1796,40 @@
     <col min="9" max="9" width="6.42578125" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="22.140625" customWidth="1"/>
     <col min="11" max="11" width="11.42578125" customWidth="1"/>
-    <col min="12" max="12" width="7.28515625" customWidth="1"/>
+    <col min="12" max="12" width="13.7109375" customWidth="1"/>
     <col min="13" max="13" width="12.42578125" customWidth="1"/>
     <col min="14" max="14" width="13.42578125" customWidth="1"/>
     <col min="15" max="15" width="20.5703125" customWidth="1"/>
     <col min="16" max="16" width="14" customWidth="1"/>
-    <col min="17" max="17" width="24.7109375" customWidth="1"/>
+    <col min="17" max="17" width="35.140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="16.5" thickBot="1">
-      <c r="A1" s="78" t="s">
+      <c r="A1" s="94" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="79"/>
-      <c r="C1" s="79"/>
-      <c r="D1" s="79"/>
-      <c r="E1" s="79"/>
-      <c r="F1" s="79"/>
-      <c r="G1" s="79"/>
-      <c r="H1" s="79"/>
-      <c r="I1" s="79"/>
-      <c r="J1" s="79"/>
-      <c r="K1" s="79"/>
-      <c r="L1" s="79"/>
-      <c r="M1" s="79"/>
-      <c r="N1" s="79"/>
-      <c r="O1" s="79"/>
-      <c r="P1" s="79"/>
-      <c r="Q1" s="80"/>
+      <c r="B1" s="95"/>
+      <c r="C1" s="95"/>
+      <c r="D1" s="95"/>
+      <c r="E1" s="95"/>
+      <c r="F1" s="95"/>
+      <c r="G1" s="95"/>
+      <c r="H1" s="95"/>
+      <c r="I1" s="95"/>
+      <c r="J1" s="95"/>
+      <c r="K1" s="95"/>
+      <c r="L1" s="95"/>
+      <c r="M1" s="95"/>
+      <c r="N1" s="95"/>
+      <c r="O1" s="95"/>
+      <c r="P1" s="95"/>
+      <c r="Q1" s="96"/>
     </row>
     <row r="2" spans="1:17" ht="16.5" thickBot="1">
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="69" t="s">
+      <c r="B2" s="61" t="s">
         <v>2</v>
       </c>
       <c r="C2" s="2" t="s">
@@ -1752,7 +1859,7 @@
       <c r="K2" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="L2" s="70" t="s">
+      <c r="L2" s="62" t="s">
         <v>12</v>
       </c>
       <c r="M2" s="2" t="s">
@@ -1764,7 +1871,7 @@
       <c r="O2" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="P2" s="71" t="s">
+      <c r="P2" s="63" t="s">
         <v>16</v>
       </c>
       <c r="Q2" s="2" t="s">
@@ -1775,491 +1882,491 @@
       <c r="A3" s="3">
         <v>1</v>
       </c>
-      <c r="B3" s="81" t="s">
+      <c r="B3" s="99" t="s">
         <v>18</v>
       </c>
       <c r="C3" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="D3" s="109" t="s">
+      <c r="D3" s="91" t="s">
         <v>137</v>
       </c>
-      <c r="E3" s="53" t="s">
+      <c r="E3" s="48" t="s">
         <v>20</v>
       </c>
-      <c r="F3" s="53" t="s">
+      <c r="F3" s="48" t="s">
         <v>21</v>
       </c>
-      <c r="G3" s="84" t="s">
+      <c r="G3" s="70" t="s">
         <v>22</v>
       </c>
       <c r="H3" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="I3" s="54" t="s">
+      <c r="I3" s="49" t="s">
         <v>24</v>
       </c>
-      <c r="J3" s="84">
+      <c r="J3" s="70">
         <v>6</v>
       </c>
-      <c r="K3" s="84">
+      <c r="K3" s="70">
         <f t="shared" ref="K3:K33" si="0">J3*5</f>
         <v>30</v>
       </c>
-      <c r="L3" s="110" t="s">
+      <c r="L3" s="92" t="s">
         <v>25</v>
       </c>
-      <c r="M3" s="104">
+      <c r="M3" s="88">
         <v>0.1</v>
       </c>
-      <c r="N3" s="105">
-        <f t="shared" ref="N3:N31" si="1">M3*J3</f>
+      <c r="N3" s="89">
+        <f>M3*J3</f>
         <v>0.60000000000000009</v>
       </c>
-      <c r="O3" s="104">
+      <c r="O3" s="88">
         <v>3.1E-2</v>
       </c>
-      <c r="P3" s="105">
-        <f t="shared" ref="P3:P31" si="2">O3*K3</f>
+      <c r="P3" s="89">
+        <f t="shared" ref="P3:P31" si="1">O3*K3</f>
         <v>0.92999999999999994</v>
       </c>
-      <c r="Q3" s="40"/>
+      <c r="Q3" s="38"/>
     </row>
     <row r="4" spans="1:17" ht="15.75" thickBot="1">
       <c r="A4" s="3">
         <v>2</v>
       </c>
-      <c r="B4" s="82"/>
-      <c r="C4" s="55" t="s">
+      <c r="B4" s="100"/>
+      <c r="C4" s="50" t="s">
         <v>138</v>
       </c>
-      <c r="D4" s="92" t="s">
+      <c r="D4" s="76" t="s">
         <v>139</v>
       </c>
-      <c r="E4" s="56" t="s">
+      <c r="E4" s="51" t="s">
         <v>20</v>
       </c>
-      <c r="F4" s="59" t="s">
+      <c r="F4" s="53" t="s">
         <v>140</v>
       </c>
-      <c r="G4" s="9" t="s">
+      <c r="G4" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="H4" s="73" t="s">
-        <v>23</v>
-      </c>
-      <c r="I4" s="74" t="s">
+      <c r="H4" s="65" t="s">
+        <v>23</v>
+      </c>
+      <c r="I4" s="66" t="s">
         <v>141</v>
       </c>
-      <c r="J4" s="9">
+      <c r="J4" s="8">
         <v>1</v>
       </c>
-      <c r="K4" s="9">
+      <c r="K4" s="8">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="L4" s="31" t="s">
+      <c r="L4" s="30" t="s">
         <v>25</v>
       </c>
-      <c r="M4" s="24">
+      <c r="M4" s="23">
         <v>0.67</v>
       </c>
-      <c r="N4" s="25">
+      <c r="N4" s="24">
+        <f t="shared" ref="N3:N31" si="2">M4*J4</f>
+        <v>0.67</v>
+      </c>
+      <c r="O4" s="23">
+        <v>0.67</v>
+      </c>
+      <c r="P4" s="24">
         <f t="shared" si="1"/>
-        <v>0.67</v>
-      </c>
-      <c r="O4" s="24">
-        <v>0.67</v>
-      </c>
-      <c r="P4" s="25">
-        <f t="shared" si="2"/>
         <v>3.35</v>
       </c>
-      <c r="Q4" s="77"/>
+      <c r="Q4" s="69"/>
     </row>
     <row r="5" spans="1:17" ht="15" customHeight="1" thickBot="1">
       <c r="A5" s="3">
         <v>3</v>
       </c>
-      <c r="B5" s="82"/>
-      <c r="C5" s="55" t="s">
+      <c r="B5" s="100"/>
+      <c r="C5" s="50" t="s">
         <v>26</v>
       </c>
-      <c r="D5" s="92" t="s">
+      <c r="D5" s="76" t="s">
         <v>27</v>
       </c>
-      <c r="E5" s="56" t="s">
+      <c r="E5" s="51" t="s">
         <v>20</v>
       </c>
-      <c r="F5" s="56" t="s">
+      <c r="F5" s="51" t="s">
         <v>28</v>
       </c>
-      <c r="G5" s="9" t="s">
+      <c r="G5" s="8" t="s">
         <v>29</v>
       </c>
-      <c r="H5" s="9" t="s">
-        <v>23</v>
-      </c>
-      <c r="I5" s="8" t="s">
+      <c r="H5" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="I5" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="J5" s="9">
+      <c r="J5" s="8">
         <v>2</v>
       </c>
-      <c r="K5" s="9">
+      <c r="K5" s="8">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="L5" s="23" t="s">
+      <c r="L5" s="22" t="s">
         <v>25</v>
       </c>
-      <c r="M5" s="24">
+      <c r="M5" s="23">
         <v>0.37</v>
       </c>
-      <c r="N5" s="25">
+      <c r="N5" s="24">
+        <f t="shared" si="2"/>
+        <v>0.74</v>
+      </c>
+      <c r="O5" s="23">
+        <v>0.25800000000000001</v>
+      </c>
+      <c r="P5" s="24">
         <f t="shared" si="1"/>
-        <v>0.74</v>
-      </c>
-      <c r="O5" s="24">
-        <v>0.25800000000000001</v>
-      </c>
-      <c r="P5" s="25">
-        <f t="shared" si="2"/>
         <v>2.58</v>
       </c>
-      <c r="Q5" s="41"/>
+      <c r="Q5" s="39"/>
     </row>
     <row r="6" spans="1:17" ht="15" customHeight="1" thickBot="1">
       <c r="A6" s="3">
         <v>4</v>
       </c>
-      <c r="B6" s="83"/>
-      <c r="C6" s="10" t="s">
+      <c r="B6" s="101"/>
+      <c r="C6" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="D6" s="93" t="s">
+      <c r="D6" s="77" t="s">
         <v>32</v>
       </c>
-      <c r="E6" s="57" t="s">
+      <c r="E6" s="52" t="s">
         <v>20</v>
       </c>
-      <c r="F6" s="57" t="s">
+      <c r="F6" s="52" t="s">
         <v>33</v>
       </c>
-      <c r="G6" s="13" t="s">
+      <c r="G6" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="H6" s="13" t="s">
-        <v>23</v>
-      </c>
-      <c r="I6" s="57" t="s">
+      <c r="H6" s="12" t="s">
+        <v>23</v>
+      </c>
+      <c r="I6" s="52" t="s">
         <v>34</v>
       </c>
-      <c r="J6" s="13">
+      <c r="J6" s="12">
         <v>2</v>
       </c>
-      <c r="K6" s="13">
+      <c r="K6" s="12">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="L6" s="26" t="s">
+      <c r="L6" s="25" t="s">
         <v>25</v>
       </c>
-      <c r="M6" s="27">
+      <c r="M6" s="26">
         <v>0.1</v>
       </c>
-      <c r="N6" s="28">
+      <c r="N6" s="27">
+        <f t="shared" si="2"/>
+        <v>0.2</v>
+      </c>
+      <c r="O6" s="26">
+        <v>3.5000000000000003E-2</v>
+      </c>
+      <c r="P6" s="27">
         <f t="shared" si="1"/>
-        <v>0.2</v>
-      </c>
-      <c r="O6" s="27">
-        <v>3.5000000000000003E-2</v>
-      </c>
-      <c r="P6" s="28">
-        <f t="shared" si="2"/>
         <v>0.35000000000000003</v>
       </c>
-      <c r="Q6" s="42"/>
+      <c r="Q6" s="40"/>
     </row>
     <row r="7" spans="1:17" ht="16.5" customHeight="1" thickBot="1">
       <c r="A7" s="3">
         <v>5</v>
       </c>
-      <c r="B7" s="81" t="s">
+      <c r="B7" s="99" t="s">
         <v>35</v>
       </c>
-      <c r="C7" s="100" t="s">
+      <c r="C7" s="84" t="s">
         <v>36</v>
       </c>
-      <c r="D7" s="101" t="s">
+      <c r="D7" s="85" t="s">
         <v>158</v>
       </c>
-      <c r="E7" s="102" t="s">
+      <c r="E7" s="86" t="s">
         <v>37</v>
       </c>
-      <c r="F7" s="102" t="s">
+      <c r="F7" s="86" t="s">
         <v>38</v>
       </c>
-      <c r="G7" s="84" t="s">
+      <c r="G7" s="70" t="s">
         <v>39</v>
       </c>
-      <c r="H7" s="84" t="s">
-        <v>23</v>
-      </c>
-      <c r="I7" s="84" t="s">
-        <v>23</v>
-      </c>
-      <c r="J7" s="84">
+      <c r="H7" s="70" t="s">
+        <v>23</v>
+      </c>
+      <c r="I7" s="70" t="s">
+        <v>23</v>
+      </c>
+      <c r="J7" s="70">
         <v>1</v>
       </c>
-      <c r="K7" s="84">
+      <c r="K7" s="70">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="L7" s="103" t="s">
+      <c r="L7" s="87" t="s">
         <v>25</v>
       </c>
-      <c r="M7" s="104">
+      <c r="M7" s="88">
         <v>0.37</v>
       </c>
-      <c r="N7" s="105">
+      <c r="N7" s="89">
+        <f t="shared" si="2"/>
+        <v>0.37</v>
+      </c>
+      <c r="O7" s="88">
+        <v>0.37</v>
+      </c>
+      <c r="P7" s="89">
         <f t="shared" si="1"/>
-        <v>0.37</v>
-      </c>
-      <c r="O7" s="104">
-        <v>0.37</v>
-      </c>
-      <c r="P7" s="105">
-        <f t="shared" si="2"/>
         <v>1.85</v>
       </c>
-      <c r="Q7" s="106"/>
+      <c r="Q7" s="90"/>
     </row>
     <row r="8" spans="1:17" ht="16.5" customHeight="1" thickBot="1">
       <c r="A8" s="3">
         <v>6</v>
       </c>
-      <c r="B8" s="82"/>
-      <c r="C8" s="55" t="s">
+      <c r="B8" s="100"/>
+      <c r="C8" s="50" t="s">
         <v>151</v>
       </c>
-      <c r="D8" s="92" t="s">
+      <c r="D8" s="76" t="s">
         <v>142</v>
       </c>
-      <c r="E8" s="56" t="s">
+      <c r="E8" s="51" t="s">
         <v>143</v>
       </c>
-      <c r="F8" s="56" t="s">
+      <c r="F8" s="51" t="s">
         <v>144</v>
       </c>
-      <c r="G8" s="9" t="s">
+      <c r="G8" s="8" t="s">
         <v>159</v>
       </c>
-      <c r="H8" s="9" t="s">
-        <v>23</v>
-      </c>
-      <c r="I8" s="9" t="s">
-        <v>23</v>
-      </c>
-      <c r="J8" s="9">
+      <c r="H8" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="I8" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="J8" s="8">
         <v>1</v>
       </c>
-      <c r="K8" s="9">
+      <c r="K8" s="8">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="L8" s="31" t="s">
+      <c r="L8" s="30" t="s">
         <v>25</v>
       </c>
-      <c r="M8" s="24">
+      <c r="M8" s="23">
         <v>0.39</v>
       </c>
-      <c r="N8" s="25">
+      <c r="N8" s="24">
+        <f t="shared" si="2"/>
+        <v>0.39</v>
+      </c>
+      <c r="O8" s="23">
+        <v>0.39</v>
+      </c>
+      <c r="P8" s="24">
         <f t="shared" si="1"/>
-        <v>0.39</v>
-      </c>
-      <c r="O8" s="24">
-        <v>0.39</v>
-      </c>
-      <c r="P8" s="25">
-        <f t="shared" si="2"/>
         <v>1.9500000000000002</v>
       </c>
-      <c r="Q8" s="41"/>
+      <c r="Q8" s="39"/>
     </row>
     <row r="9" spans="1:17" ht="16.5" customHeight="1" thickBot="1">
       <c r="A9" s="3">
         <v>7</v>
       </c>
-      <c r="B9" s="82"/>
-      <c r="C9" s="97" t="s">
+      <c r="B9" s="100"/>
+      <c r="C9" s="81" t="s">
         <v>160</v>
       </c>
-      <c r="D9" s="96" t="s">
+      <c r="D9" s="80" t="s">
         <v>145</v>
       </c>
-      <c r="E9" s="74" t="s">
+      <c r="E9" s="66" t="s">
         <v>143</v>
       </c>
-      <c r="F9" s="63" t="s">
+      <c r="F9" s="57" t="s">
         <v>146</v>
       </c>
-      <c r="G9" s="9" t="s">
+      <c r="G9" s="8" t="s">
         <v>159</v>
       </c>
-      <c r="H9" s="73" t="s">
-        <v>23</v>
-      </c>
-      <c r="I9" s="73" t="s">
-        <v>23</v>
-      </c>
-      <c r="J9" s="73">
+      <c r="H9" s="65" t="s">
+        <v>23</v>
+      </c>
+      <c r="I9" s="65" t="s">
+        <v>23</v>
+      </c>
+      <c r="J9" s="65">
         <v>1</v>
       </c>
-      <c r="K9" s="9">
+      <c r="K9" s="8">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="L9" s="31" t="s">
+      <c r="L9" s="30" t="s">
         <v>25</v>
       </c>
-      <c r="M9" s="24">
+      <c r="M9" s="23">
         <v>0.52</v>
       </c>
-      <c r="N9" s="25">
+      <c r="N9" s="24">
+        <f t="shared" si="2"/>
+        <v>0.52</v>
+      </c>
+      <c r="O9" s="23">
+        <v>0.52</v>
+      </c>
+      <c r="P9" s="24">
         <f t="shared" si="1"/>
-        <v>0.52</v>
-      </c>
-      <c r="O9" s="24">
-        <v>0.52</v>
-      </c>
-      <c r="P9" s="25">
-        <f t="shared" si="2"/>
         <v>2.6</v>
       </c>
-      <c r="Q9" s="41"/>
+      <c r="Q9" s="39"/>
     </row>
     <row r="10" spans="1:17" ht="16.5" customHeight="1" thickBot="1">
       <c r="A10" s="3">
         <v>8</v>
       </c>
-      <c r="B10" s="82"/>
-      <c r="C10" s="55" t="s">
+      <c r="B10" s="100"/>
+      <c r="C10" s="50" t="s">
         <v>161</v>
       </c>
-      <c r="D10" s="92" t="s">
+      <c r="D10" s="76" t="s">
         <v>147</v>
       </c>
-      <c r="E10" s="56" t="s">
+      <c r="E10" s="51" t="s">
         <v>143</v>
       </c>
-      <c r="F10" s="59" t="s">
+      <c r="F10" s="53" t="s">
         <v>148</v>
       </c>
-      <c r="G10" s="9" t="s">
+      <c r="G10" s="8" t="s">
         <v>159</v>
       </c>
-      <c r="H10" s="9" t="s">
-        <v>23</v>
-      </c>
-      <c r="I10" s="9" t="s">
-        <v>23</v>
-      </c>
-      <c r="J10" s="9">
+      <c r="H10" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="I10" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="J10" s="8">
         <v>1</v>
       </c>
-      <c r="K10" s="9">
+      <c r="K10" s="8">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="L10" s="31" t="s">
+      <c r="L10" s="30" t="s">
         <v>25</v>
       </c>
-      <c r="M10" s="24">
+      <c r="M10" s="23">
         <v>0.25</v>
       </c>
-      <c r="N10" s="25">
+      <c r="N10" s="24">
+        <f t="shared" si="2"/>
+        <v>0.25</v>
+      </c>
+      <c r="O10" s="23">
+        <v>0.25</v>
+      </c>
+      <c r="P10" s="24">
         <f t="shared" si="1"/>
-        <v>0.25</v>
-      </c>
-      <c r="O10" s="24">
-        <v>0.25</v>
-      </c>
-      <c r="P10" s="25">
-        <f t="shared" si="2"/>
         <v>1.25</v>
       </c>
-      <c r="Q10" s="41"/>
+      <c r="Q10" s="39"/>
     </row>
     <row r="11" spans="1:17" ht="16.5" customHeight="1" thickBot="1">
       <c r="A11" s="3">
         <v>9</v>
       </c>
-      <c r="B11" s="83"/>
-      <c r="C11" s="111" t="s">
+      <c r="B11" s="101"/>
+      <c r="C11" s="93" t="s">
         <v>162</v>
       </c>
-      <c r="D11" s="93" t="s">
+      <c r="D11" s="77" t="s">
         <v>149</v>
       </c>
-      <c r="E11" s="57" t="s">
+      <c r="E11" s="52" t="s">
         <v>143</v>
       </c>
-      <c r="F11" s="57" t="s">
+      <c r="F11" s="52" t="s">
         <v>150</v>
       </c>
-      <c r="G11" s="13" t="s">
+      <c r="G11" s="12" t="s">
         <v>159</v>
       </c>
-      <c r="H11" s="13" t="s">
-        <v>23</v>
-      </c>
-      <c r="I11" s="13" t="s">
-        <v>23</v>
-      </c>
-      <c r="J11" s="13">
+      <c r="H11" s="12" t="s">
+        <v>23</v>
+      </c>
+      <c r="I11" s="12" t="s">
+        <v>23</v>
+      </c>
+      <c r="J11" s="12">
         <v>1</v>
       </c>
-      <c r="K11" s="13">
+      <c r="K11" s="12">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="L11" s="26" t="s">
+      <c r="L11" s="25" t="s">
         <v>25</v>
       </c>
-      <c r="M11" s="27">
+      <c r="M11" s="26">
         <v>0.37</v>
       </c>
-      <c r="N11" s="28">
+      <c r="N11" s="27">
+        <f t="shared" si="2"/>
+        <v>0.37</v>
+      </c>
+      <c r="O11" s="26">
+        <v>0.37</v>
+      </c>
+      <c r="P11" s="27">
         <f t="shared" si="1"/>
-        <v>0.37</v>
-      </c>
-      <c r="O11" s="27">
-        <v>0.37</v>
-      </c>
-      <c r="P11" s="28">
-        <f t="shared" si="2"/>
         <v>1.85</v>
       </c>
-      <c r="Q11" s="42"/>
+      <c r="Q11" s="40"/>
     </row>
     <row r="12" spans="1:17" ht="15.75" thickBot="1">
       <c r="A12" s="3">
         <v>10</v>
       </c>
-      <c r="B12" s="81" t="s">
+      <c r="B12" s="99" t="s">
         <v>40</v>
       </c>
-      <c r="C12" s="98" t="s">
+      <c r="C12" s="82" t="s">
         <v>41</v>
       </c>
-      <c r="D12" s="99" t="s">
+      <c r="D12" s="83" t="s">
         <v>42</v>
       </c>
-      <c r="E12" s="53" t="s">
+      <c r="E12" s="48" t="s">
         <v>43</v>
       </c>
-      <c r="F12" s="53" t="s">
+      <c r="F12" s="48" t="s">
         <v>44</v>
       </c>
       <c r="G12" s="5" t="s">
@@ -2278,146 +2385,146 @@
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="L12" s="30" t="s">
+      <c r="L12" s="29" t="s">
         <v>25</v>
       </c>
-      <c r="M12" s="21">
+      <c r="M12" s="20">
         <v>0.44</v>
       </c>
-      <c r="N12" s="22">
+      <c r="N12" s="21">
+        <f t="shared" si="2"/>
+        <v>0.44</v>
+      </c>
+      <c r="O12" s="20">
+        <v>0.44</v>
+      </c>
+      <c r="P12" s="21">
         <f t="shared" si="1"/>
-        <v>0.44</v>
-      </c>
-      <c r="O12" s="21">
-        <v>0.44</v>
-      </c>
-      <c r="P12" s="22">
-        <f t="shared" si="2"/>
         <v>2.2000000000000002</v>
       </c>
-      <c r="Q12" s="40"/>
+      <c r="Q12" s="38"/>
     </row>
     <row r="13" spans="1:17" ht="15" customHeight="1" thickBot="1">
       <c r="A13" s="3">
         <v>11</v>
       </c>
-      <c r="B13" s="82"/>
+      <c r="B13" s="100"/>
       <c r="C13" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="D13" s="92" t="s">
+      <c r="D13" s="76" t="s">
         <v>47</v>
       </c>
-      <c r="E13" s="56" t="s">
+      <c r="E13" s="51" t="s">
         <v>48</v>
       </c>
-      <c r="F13" s="56" t="s">
+      <c r="F13" s="51" t="s">
         <v>49</v>
       </c>
-      <c r="G13" s="9" t="s">
+      <c r="G13" s="8" t="s">
         <v>45</v>
       </c>
-      <c r="H13" s="9" t="s">
-        <v>23</v>
-      </c>
-      <c r="I13" s="9" t="s">
-        <v>23</v>
-      </c>
-      <c r="J13" s="9">
+      <c r="H13" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="I13" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="J13" s="8">
         <v>2</v>
       </c>
-      <c r="K13" s="9">
+      <c r="K13" s="8">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="L13" s="31" t="s">
+      <c r="L13" s="30" t="s">
         <v>25</v>
       </c>
-      <c r="M13" s="24">
+      <c r="M13" s="23">
         <v>0.14000000000000001</v>
       </c>
-      <c r="N13" s="25">
+      <c r="N13" s="24">
+        <f t="shared" si="2"/>
+        <v>0.28000000000000003</v>
+      </c>
+      <c r="O13" s="23">
+        <v>0.13200000000000001</v>
+      </c>
+      <c r="P13" s="24">
         <f t="shared" si="1"/>
-        <v>0.28000000000000003</v>
-      </c>
-      <c r="O13" s="24">
-        <v>0.13200000000000001</v>
-      </c>
-      <c r="P13" s="25">
-        <f t="shared" si="2"/>
         <v>1.32</v>
       </c>
-      <c r="Q13" s="41"/>
+      <c r="Q13" s="39"/>
     </row>
     <row r="14" spans="1:17" ht="15" customHeight="1" thickBot="1">
       <c r="A14" s="3">
         <v>12</v>
       </c>
-      <c r="B14" s="83"/>
-      <c r="C14" s="10" t="s">
+      <c r="B14" s="101"/>
+      <c r="C14" s="9" t="s">
         <v>154</v>
       </c>
-      <c r="D14" s="11" t="s">
+      <c r="D14" s="10" t="s">
         <v>155</v>
       </c>
-      <c r="E14" s="57" t="s">
+      <c r="E14" s="52" t="s">
         <v>156</v>
       </c>
-      <c r="F14" s="57" t="s">
+      <c r="F14" s="52" t="s">
         <v>157</v>
       </c>
-      <c r="G14" s="13" t="s">
+      <c r="G14" s="12" t="s">
         <v>45</v>
       </c>
-      <c r="H14" s="13" t="s">
-        <v>23</v>
-      </c>
-      <c r="I14" s="13" t="s">
-        <v>23</v>
-      </c>
-      <c r="J14" s="13">
+      <c r="H14" s="12" t="s">
+        <v>23</v>
+      </c>
+      <c r="I14" s="12" t="s">
+        <v>23</v>
+      </c>
+      <c r="J14" s="12">
         <v>1</v>
       </c>
-      <c r="K14" s="13">
+      <c r="K14" s="12">
         <f>J14*5</f>
         <v>5</v>
       </c>
-      <c r="L14" s="26" t="s">
+      <c r="L14" s="25" t="s">
         <v>25</v>
       </c>
-      <c r="M14" s="27">
+      <c r="M14" s="26">
         <v>0.55000000000000004</v>
       </c>
-      <c r="N14" s="28">
+      <c r="N14" s="27">
         <f>M14*J14</f>
         <v>0.55000000000000004</v>
       </c>
-      <c r="O14" s="27">
+      <c r="O14" s="26">
         <v>0.55000000000000004</v>
       </c>
-      <c r="P14" s="28">
+      <c r="P14" s="27">
         <f>O14*K14</f>
         <v>2.75</v>
       </c>
-      <c r="Q14" s="42"/>
+      <c r="Q14" s="40"/>
     </row>
     <row r="15" spans="1:17" ht="16.5" customHeight="1" thickBot="1">
       <c r="A15" s="3">
         <v>13</v>
       </c>
-      <c r="B15" s="81" t="s">
+      <c r="B15" s="99" t="s">
         <v>50</v>
       </c>
       <c r="C15" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="D15" s="94" t="s">
+      <c r="D15" s="78" t="s">
         <v>52</v>
       </c>
-      <c r="E15" s="54" t="s">
+      <c r="E15" s="49" t="s">
         <v>53</v>
       </c>
-      <c r="F15" s="54" t="s">
+      <c r="F15" s="49" t="s">
         <v>54</v>
       </c>
       <c r="G15" s="5" t="s">
@@ -2426,912 +2533,910 @@
       <c r="H15" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="I15" s="54" t="s">
+      <c r="I15" s="49" t="s">
         <v>56</v>
       </c>
-      <c r="J15" s="14">
+      <c r="J15" s="13">
         <v>5</v>
       </c>
       <c r="K15" s="5">
         <f t="shared" si="0"/>
         <v>25</v>
       </c>
-      <c r="L15" s="30" t="s">
+      <c r="L15" s="29" t="s">
         <v>25</v>
       </c>
-      <c r="M15" s="21">
+      <c r="M15" s="20">
         <v>0.1</v>
       </c>
-      <c r="N15" s="22">
+      <c r="N15" s="21">
+        <f t="shared" si="2"/>
+        <v>0.5</v>
+      </c>
+      <c r="O15" s="20">
+        <v>5.8000000000000003E-2</v>
+      </c>
+      <c r="P15" s="21">
         <f t="shared" si="1"/>
-        <v>0.5</v>
-      </c>
-      <c r="O15" s="21">
-        <v>5.8000000000000003E-2</v>
-      </c>
-      <c r="P15" s="22">
-        <f t="shared" si="2"/>
         <v>1.4500000000000002</v>
       </c>
-      <c r="Q15" s="40"/>
+      <c r="Q15" s="38"/>
     </row>
     <row r="16" spans="1:17" ht="15" customHeight="1" thickBot="1">
       <c r="A16" s="3">
         <v>14</v>
       </c>
-      <c r="B16" s="82"/>
-      <c r="C16" s="60" t="s">
+      <c r="B16" s="100"/>
+      <c r="C16" s="54" t="s">
         <v>57</v>
       </c>
-      <c r="D16" s="92" t="s">
+      <c r="D16" s="76" t="s">
         <v>58</v>
       </c>
-      <c r="E16" s="8" t="s">
+      <c r="E16" s="7" t="s">
         <v>59</v>
       </c>
-      <c r="F16" s="56" t="s">
+      <c r="F16" s="51" t="s">
         <v>60</v>
       </c>
-      <c r="G16" s="9" t="s">
+      <c r="G16" s="8" t="s">
         <v>61</v>
       </c>
-      <c r="H16" s="9" t="s">
-        <v>23</v>
-      </c>
-      <c r="I16" s="56" t="s">
+      <c r="H16" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="I16" s="51" t="s">
         <v>56</v>
       </c>
-      <c r="J16" s="8">
+      <c r="J16" s="7">
         <v>1</v>
       </c>
-      <c r="K16" s="9">
+      <c r="K16" s="8">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="L16" s="31" t="s">
+      <c r="L16" s="30" t="s">
         <v>25</v>
       </c>
-      <c r="M16" s="24">
+      <c r="M16" s="23">
         <v>0.26</v>
       </c>
-      <c r="N16" s="25">
+      <c r="N16" s="24">
+        <f t="shared" si="2"/>
+        <v>0.26</v>
+      </c>
+      <c r="O16" s="23">
+        <v>0.26</v>
+      </c>
+      <c r="P16" s="24">
         <f t="shared" si="1"/>
-        <v>0.26</v>
-      </c>
-      <c r="O16" s="24">
-        <v>0.26</v>
-      </c>
-      <c r="P16" s="25">
-        <f t="shared" si="2"/>
         <v>1.3</v>
       </c>
-      <c r="Q16" s="41"/>
+      <c r="Q16" s="39"/>
     </row>
     <row r="17" spans="1:17" ht="15" customHeight="1" thickBot="1">
       <c r="A17" s="3">
         <v>15</v>
       </c>
-      <c r="B17" s="82"/>
-      <c r="C17" s="60" t="s">
+      <c r="B17" s="100"/>
+      <c r="C17" s="54" t="s">
         <v>62</v>
       </c>
-      <c r="D17" s="92" t="s">
+      <c r="D17" s="76" t="s">
         <v>63</v>
       </c>
-      <c r="E17" s="56" t="s">
+      <c r="E17" s="51" t="s">
         <v>53</v>
       </c>
-      <c r="F17" s="56" t="s">
+      <c r="F17" s="51" t="s">
         <v>64</v>
       </c>
-      <c r="G17" s="9" t="s">
+      <c r="G17" s="8" t="s">
         <v>65</v>
       </c>
-      <c r="H17" s="9" t="s">
-        <v>23</v>
-      </c>
-      <c r="I17" s="56" t="s">
+      <c r="H17" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="I17" s="51" t="s">
         <v>66</v>
       </c>
-      <c r="J17" s="8">
+      <c r="J17" s="7">
         <v>2</v>
       </c>
-      <c r="K17" s="9">
+      <c r="K17" s="8">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="L17" s="31" t="s">
+      <c r="L17" s="30" t="s">
         <v>25</v>
       </c>
-      <c r="M17" s="24">
+      <c r="M17" s="23">
         <v>0.1</v>
       </c>
-      <c r="N17" s="25">
+      <c r="N17" s="24">
+        <f t="shared" si="2"/>
+        <v>0.2</v>
+      </c>
+      <c r="O17" s="23">
+        <v>0.1</v>
+      </c>
+      <c r="P17" s="24">
         <f t="shared" si="1"/>
-        <v>0.2</v>
-      </c>
-      <c r="O17" s="24">
-        <v>0.1</v>
-      </c>
-      <c r="P17" s="25">
-        <f t="shared" si="2"/>
         <v>1</v>
       </c>
-      <c r="Q17" s="41"/>
+      <c r="Q17" s="39"/>
     </row>
     <row r="18" spans="1:17" ht="15" customHeight="1" thickBot="1">
       <c r="A18" s="3">
         <v>16</v>
       </c>
-      <c r="B18" s="82"/>
+      <c r="B18" s="100"/>
       <c r="C18" s="6" t="s">
         <v>67</v>
       </c>
-      <c r="D18" s="92" t="s">
+      <c r="D18" s="76" t="s">
         <v>68</v>
       </c>
-      <c r="E18" s="56" t="s">
+      <c r="E18" s="51" t="s">
         <v>53</v>
       </c>
-      <c r="F18" s="56" t="s">
+      <c r="F18" s="51" t="s">
         <v>69</v>
       </c>
-      <c r="G18" s="9" t="s">
+      <c r="G18" s="8" t="s">
         <v>65</v>
       </c>
-      <c r="H18" s="15" t="s">
-        <v>23</v>
-      </c>
-      <c r="I18" s="56" t="s">
+      <c r="H18" s="14" t="s">
+        <v>23</v>
+      </c>
+      <c r="I18" s="51" t="s">
         <v>70</v>
       </c>
-      <c r="J18" s="8">
+      <c r="J18" s="7">
         <v>1</v>
       </c>
-      <c r="K18" s="9">
+      <c r="K18" s="8">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="L18" s="31" t="s">
+      <c r="L18" s="30" t="s">
         <v>25</v>
       </c>
-      <c r="M18" s="24">
+      <c r="M18" s="23">
         <v>0.1</v>
       </c>
-      <c r="N18" s="25">
+      <c r="N18" s="24">
+        <f t="shared" si="2"/>
+        <v>0.1</v>
+      </c>
+      <c r="O18" s="23">
+        <v>0.1</v>
+      </c>
+      <c r="P18" s="24">
         <f t="shared" si="1"/>
-        <v>0.1</v>
-      </c>
-      <c r="O18" s="24">
-        <v>0.1</v>
-      </c>
-      <c r="P18" s="25">
-        <f t="shared" si="2"/>
         <v>0.5</v>
       </c>
-      <c r="Q18" s="41"/>
+      <c r="Q18" s="39"/>
     </row>
     <row r="19" spans="1:17" ht="15" customHeight="1" thickBot="1">
       <c r="A19" s="3">
         <v>17</v>
       </c>
-      <c r="B19" s="82"/>
+      <c r="B19" s="100"/>
       <c r="C19" s="6" t="s">
         <v>71</v>
       </c>
-      <c r="D19" s="92" t="s">
+      <c r="D19" s="76" t="s">
         <v>152</v>
       </c>
-      <c r="E19" s="56" t="s">
+      <c r="E19" s="51" t="s">
         <v>53</v>
       </c>
-      <c r="F19" s="56" t="s">
+      <c r="F19" s="51" t="s">
         <v>72</v>
       </c>
-      <c r="G19" s="9" t="s">
+      <c r="G19" s="8" t="s">
         <v>65</v>
       </c>
-      <c r="H19" s="9" t="s">
-        <v>23</v>
-      </c>
-      <c r="I19" s="56" t="s">
+      <c r="H19" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="I19" s="51" t="s">
         <v>73</v>
       </c>
-      <c r="J19" s="8">
+      <c r="J19" s="7">
         <v>4</v>
       </c>
-      <c r="K19" s="9">
+      <c r="K19" s="8">
         <f t="shared" si="0"/>
         <v>20</v>
       </c>
-      <c r="L19" s="31" t="s">
+      <c r="L19" s="30" t="s">
         <v>25</v>
       </c>
-      <c r="M19" s="25">
+      <c r="M19" s="24">
         <v>0.1</v>
       </c>
-      <c r="N19" s="25">
+      <c r="N19" s="24">
+        <f t="shared" si="2"/>
+        <v>0.4</v>
+      </c>
+      <c r="O19" s="24">
+        <v>2.4E-2</v>
+      </c>
+      <c r="P19" s="24">
         <f t="shared" si="1"/>
-        <v>0.4</v>
-      </c>
-      <c r="O19" s="25">
-        <v>2.4E-2</v>
-      </c>
-      <c r="P19" s="25">
-        <f t="shared" si="2"/>
         <v>0.48</v>
       </c>
-      <c r="Q19" s="43"/>
+      <c r="Q19" s="41"/>
     </row>
     <row r="20" spans="1:17" ht="15" customHeight="1" thickBot="1">
       <c r="A20" s="3">
         <v>18</v>
       </c>
-      <c r="B20" s="82"/>
-      <c r="C20" s="60" t="s">
+      <c r="B20" s="100"/>
+      <c r="C20" s="54" t="s">
         <v>74</v>
       </c>
-      <c r="D20" s="92" t="s">
+      <c r="D20" s="76" t="s">
         <v>75</v>
       </c>
-      <c r="E20" s="56" t="s">
+      <c r="E20" s="51" t="s">
         <v>53</v>
       </c>
-      <c r="F20" s="56" t="s">
+      <c r="F20" s="51" t="s">
         <v>76</v>
       </c>
-      <c r="G20" s="9" t="s">
+      <c r="G20" s="8" t="s">
         <v>77</v>
       </c>
-      <c r="H20" s="9" t="s">
-        <v>23</v>
-      </c>
-      <c r="I20" s="8" t="s">
+      <c r="H20" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="I20" s="7" t="s">
         <v>78</v>
       </c>
-      <c r="J20" s="8">
+      <c r="J20" s="7">
         <v>1</v>
       </c>
-      <c r="K20" s="9">
+      <c r="K20" s="8">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="L20" s="31" t="s">
+      <c r="L20" s="30" t="s">
         <v>25</v>
       </c>
-      <c r="M20" s="25">
+      <c r="M20" s="24">
         <v>0.1</v>
       </c>
-      <c r="N20" s="25">
+      <c r="N20" s="24">
+        <f t="shared" si="2"/>
+        <v>0.1</v>
+      </c>
+      <c r="O20" s="24">
+        <v>0.1</v>
+      </c>
+      <c r="P20" s="24">
         <f t="shared" si="1"/>
-        <v>0.1</v>
-      </c>
-      <c r="O20" s="25">
-        <v>0.1</v>
-      </c>
-      <c r="P20" s="25">
-        <f t="shared" si="2"/>
         <v>0.5</v>
       </c>
-      <c r="Q20" s="43"/>
+      <c r="Q20" s="41"/>
     </row>
     <row r="21" spans="1:17" ht="15" customHeight="1" thickBot="1">
       <c r="A21" s="3">
         <v>19</v>
       </c>
-      <c r="B21" s="82"/>
-      <c r="C21" s="60" t="s">
+      <c r="B21" s="100"/>
+      <c r="C21" s="54" t="s">
         <v>79</v>
       </c>
-      <c r="D21" s="92" t="s">
+      <c r="D21" s="76" t="s">
         <v>80</v>
       </c>
-      <c r="E21" s="56" t="s">
+      <c r="E21" s="51" t="s">
         <v>53</v>
       </c>
-      <c r="F21" s="56" t="s">
+      <c r="F21" s="51" t="s">
         <v>81</v>
       </c>
-      <c r="G21" s="9" t="s">
+      <c r="G21" s="8" t="s">
         <v>82</v>
       </c>
-      <c r="H21" s="9" t="s">
-        <v>23</v>
-      </c>
-      <c r="I21" s="8" t="s">
+      <c r="H21" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="I21" s="7" t="s">
         <v>83</v>
       </c>
-      <c r="J21" s="8">
+      <c r="J21" s="7">
         <v>1</v>
       </c>
-      <c r="K21" s="9">
+      <c r="K21" s="8">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="L21" s="31" t="s">
+      <c r="L21" s="30" t="s">
         <v>25</v>
       </c>
-      <c r="M21" s="25">
+      <c r="M21" s="24">
         <v>0.1</v>
       </c>
-      <c r="N21" s="25">
+      <c r="N21" s="24">
+        <f t="shared" si="2"/>
+        <v>0.1</v>
+      </c>
+      <c r="O21" s="24">
+        <v>0.1</v>
+      </c>
+      <c r="P21" s="24">
         <f t="shared" si="1"/>
-        <v>0.1</v>
-      </c>
-      <c r="O21" s="25">
-        <v>0.1</v>
-      </c>
-      <c r="P21" s="25">
-        <f t="shared" si="2"/>
         <v>0.5</v>
       </c>
-      <c r="Q21" s="43"/>
+      <c r="Q21" s="41"/>
     </row>
     <row r="22" spans="1:17" ht="15" customHeight="1" thickBot="1">
       <c r="A22" s="3">
         <v>20</v>
       </c>
-      <c r="B22" s="82"/>
+      <c r="B22" s="100"/>
       <c r="C22" s="6" t="s">
         <v>84</v>
       </c>
-      <c r="D22" s="92" t="s">
+      <c r="D22" s="76" t="s">
         <v>85</v>
       </c>
-      <c r="E22" s="56" t="s">
+      <c r="E22" s="51" t="s">
         <v>53</v>
       </c>
-      <c r="F22" s="56" t="s">
+      <c r="F22" s="51" t="s">
         <v>86</v>
       </c>
-      <c r="G22" s="9" t="s">
+      <c r="G22" s="8" t="s">
         <v>65</v>
       </c>
-      <c r="H22" s="9" t="s">
-        <v>23</v>
-      </c>
-      <c r="I22" s="8" t="s">
+      <c r="H22" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="I22" s="7" t="s">
         <v>87</v>
       </c>
-      <c r="J22" s="8">
+      <c r="J22" s="7">
         <v>1</v>
       </c>
-      <c r="K22" s="9">
+      <c r="K22" s="8">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="L22" s="31" t="s">
+      <c r="L22" s="30" t="s">
         <v>25</v>
       </c>
-      <c r="M22" s="25">
+      <c r="M22" s="24">
         <v>0.1</v>
       </c>
-      <c r="N22" s="25">
+      <c r="N22" s="24">
+        <f t="shared" si="2"/>
+        <v>0.1</v>
+      </c>
+      <c r="O22" s="24">
+        <v>0.1</v>
+      </c>
+      <c r="P22" s="24">
         <f t="shared" si="1"/>
-        <v>0.1</v>
-      </c>
-      <c r="O22" s="25">
-        <v>0.1</v>
-      </c>
-      <c r="P22" s="25">
-        <f t="shared" si="2"/>
         <v>0.5</v>
       </c>
-      <c r="Q22" s="43"/>
+      <c r="Q22" s="41"/>
     </row>
     <row r="23" spans="1:17" ht="15" customHeight="1" thickBot="1">
       <c r="A23" s="3">
         <v>21</v>
       </c>
-      <c r="B23" s="82"/>
-      <c r="C23" s="60" t="s">
+      <c r="B23" s="100"/>
+      <c r="C23" s="54" t="s">
         <v>88</v>
       </c>
-      <c r="D23" s="92" t="s">
+      <c r="D23" s="76" t="s">
         <v>89</v>
       </c>
-      <c r="E23" s="56" t="s">
+      <c r="E23" s="51" t="s">
         <v>53</v>
       </c>
-      <c r="F23" s="56" t="s">
+      <c r="F23" s="51" t="s">
         <v>90</v>
       </c>
-      <c r="G23" s="9" t="s">
+      <c r="G23" s="8" t="s">
         <v>65</v>
       </c>
-      <c r="H23" s="9" t="s">
-        <v>23</v>
-      </c>
-      <c r="I23" s="8" t="s">
+      <c r="H23" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="I23" s="7" t="s">
         <v>91</v>
       </c>
-      <c r="J23" s="8">
+      <c r="J23" s="7">
         <v>1</v>
       </c>
-      <c r="K23" s="9">
+      <c r="K23" s="8">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="L23" s="31" t="s">
+      <c r="L23" s="30" t="s">
         <v>25</v>
       </c>
-      <c r="M23" s="25">
+      <c r="M23" s="24">
         <v>0.1</v>
       </c>
-      <c r="N23" s="25">
+      <c r="N23" s="24">
+        <f t="shared" si="2"/>
+        <v>0.1</v>
+      </c>
+      <c r="O23" s="24">
+        <v>0.1</v>
+      </c>
+      <c r="P23" s="24">
         <f t="shared" si="1"/>
-        <v>0.1</v>
-      </c>
-      <c r="O23" s="25">
-        <v>0.1</v>
-      </c>
-      <c r="P23" s="25">
-        <f t="shared" si="2"/>
         <v>0.5</v>
       </c>
-      <c r="Q23" s="43"/>
+      <c r="Q23" s="41"/>
     </row>
     <row r="24" spans="1:17" ht="15.75" thickBot="1">
       <c r="A24" s="3">
         <v>22</v>
       </c>
-      <c r="B24" s="83"/>
-      <c r="C24" s="10" t="s">
+      <c r="B24" s="101"/>
+      <c r="C24" s="9" t="s">
         <v>92</v>
       </c>
-      <c r="D24" s="93" t="s">
+      <c r="D24" s="77" t="s">
         <v>93</v>
       </c>
-      <c r="E24" s="57" t="s">
+      <c r="E24" s="52" t="s">
         <v>53</v>
       </c>
-      <c r="F24" s="57" t="s">
+      <c r="F24" s="52" t="s">
         <v>94</v>
       </c>
-      <c r="G24" s="13" t="s">
+      <c r="G24" s="12" t="s">
         <v>65</v>
       </c>
-      <c r="H24" s="13" t="s">
-        <v>23</v>
-      </c>
-      <c r="I24" s="12" t="s">
+      <c r="H24" s="12" t="s">
+        <v>23</v>
+      </c>
+      <c r="I24" s="11" t="s">
         <v>95</v>
       </c>
-      <c r="J24" s="12">
+      <c r="J24" s="11">
         <v>4</v>
       </c>
-      <c r="K24" s="13">
+      <c r="K24" s="12">
         <f t="shared" si="0"/>
         <v>20</v>
       </c>
-      <c r="L24" s="26" t="s">
+      <c r="L24" s="25" t="s">
         <v>25</v>
       </c>
-      <c r="M24" s="28">
+      <c r="M24" s="27">
         <v>0.1</v>
       </c>
-      <c r="N24" s="28">
+      <c r="N24" s="27">
+        <f t="shared" si="2"/>
+        <v>0.4</v>
+      </c>
+      <c r="O24" s="27">
+        <v>0.1</v>
+      </c>
+      <c r="P24" s="27">
         <f t="shared" si="1"/>
-        <v>0.4</v>
-      </c>
-      <c r="O24" s="28">
-        <v>0.1</v>
-      </c>
-      <c r="P24" s="28">
-        <f t="shared" si="2"/>
         <v>2</v>
       </c>
-      <c r="Q24" s="44"/>
+      <c r="Q24" s="42"/>
     </row>
     <row r="25" spans="1:17" ht="16.5" thickBot="1">
       <c r="A25" s="3">
         <v>23</v>
       </c>
-      <c r="B25" s="72" t="s">
+      <c r="B25" s="64" t="s">
         <v>96</v>
       </c>
-      <c r="C25" s="61" t="s">
+      <c r="C25" s="55" t="s">
         <v>97</v>
       </c>
-      <c r="D25" s="62" t="s">
+      <c r="D25" s="56" t="s">
         <v>98</v>
       </c>
-      <c r="E25" s="16" t="s">
+      <c r="E25" s="15" t="s">
         <v>59</v>
       </c>
-      <c r="F25" s="63" t="s">
+      <c r="F25" s="57" t="s">
         <v>99</v>
       </c>
-      <c r="G25" s="17"/>
-      <c r="H25" s="17"/>
-      <c r="I25" s="17" t="s">
-        <v>23</v>
-      </c>
-      <c r="J25" s="17">
+      <c r="G25" s="16"/>
+      <c r="H25" s="16"/>
+      <c r="I25" s="16" t="s">
+        <v>23</v>
+      </c>
+      <c r="J25" s="16">
         <v>1</v>
       </c>
-      <c r="K25" s="17">
+      <c r="K25" s="16">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="L25" s="32"/>
-      <c r="M25" s="29"/>
-      <c r="N25" s="29">
+      <c r="L25" s="31"/>
+      <c r="M25" s="28"/>
+      <c r="N25" s="28">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="O25" s="28"/>
+      <c r="P25" s="28">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="O25" s="29"/>
-      <c r="P25" s="29">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="Q25" s="45"/>
+      <c r="Q25" s="43"/>
     </row>
     <row r="26" spans="1:17" ht="16.5" thickBot="1">
       <c r="A26" s="3">
         <v>24</v>
       </c>
-      <c r="B26" s="18" t="s">
+      <c r="B26" s="17" t="s">
         <v>100</v>
       </c>
-      <c r="C26" s="64" t="s">
+      <c r="C26" s="58" t="s">
         <v>101</v>
       </c>
-      <c r="D26" s="95" t="s">
+      <c r="D26" s="79" t="s">
         <v>102</v>
       </c>
-      <c r="E26" s="19" t="s">
+      <c r="E26" s="18" t="s">
         <v>59</v>
       </c>
-      <c r="F26" s="65" t="s">
+      <c r="F26" s="59" t="s">
         <v>103</v>
       </c>
-      <c r="G26" s="20" t="s">
+      <c r="G26" s="19" t="s">
         <v>104</v>
       </c>
-      <c r="H26" s="20" t="s">
-        <v>23</v>
-      </c>
-      <c r="I26" s="20" t="s">
-        <v>23</v>
-      </c>
-      <c r="J26" s="20">
+      <c r="H26" s="19" t="s">
+        <v>23</v>
+      </c>
+      <c r="I26" s="19" t="s">
+        <v>23</v>
+      </c>
+      <c r="J26" s="19">
         <v>2</v>
       </c>
-      <c r="K26" s="20">
+      <c r="K26" s="19">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="L26" s="33" t="s">
+      <c r="L26" s="32" t="s">
         <v>25</v>
       </c>
-      <c r="M26" s="34">
+      <c r="M26" s="33">
         <v>0.96</v>
       </c>
-      <c r="N26" s="35">
+      <c r="N26" s="34">
+        <f t="shared" si="2"/>
+        <v>1.92</v>
+      </c>
+      <c r="O26" s="34">
+        <v>0.92700000000000005</v>
+      </c>
+      <c r="P26" s="34">
         <f t="shared" si="1"/>
-        <v>1.92</v>
-      </c>
-      <c r="O26" s="35">
-        <v>0.92700000000000005</v>
-      </c>
-      <c r="P26" s="35">
-        <f t="shared" si="2"/>
         <v>9.27</v>
       </c>
-      <c r="Q26" s="46"/>
+      <c r="Q26" s="44"/>
     </row>
     <row r="27" spans="1:17" ht="15" customHeight="1" thickBot="1">
       <c r="A27" s="3">
         <v>25</v>
       </c>
-      <c r="B27" s="81" t="s">
+      <c r="B27" s="99" t="s">
         <v>105</v>
       </c>
-      <c r="C27" s="58" t="s">
+      <c r="C27" s="104" t="s">
         <v>106</v>
       </c>
-      <c r="D27" s="94" t="s">
+      <c r="D27" s="105" t="s">
         <v>107</v>
       </c>
-      <c r="E27" s="14" t="s">
+      <c r="E27" s="106" t="s">
         <v>59</v>
       </c>
-      <c r="F27" s="54" t="s">
+      <c r="F27" s="105" t="s">
         <v>153</v>
       </c>
-      <c r="G27" s="5" t="s">
+      <c r="G27" s="107" t="s">
         <v>108</v>
       </c>
-      <c r="H27" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="I27" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="J27" s="14">
+      <c r="H27" s="107" t="s">
+        <v>23</v>
+      </c>
+      <c r="I27" s="107" t="s">
+        <v>23</v>
+      </c>
+      <c r="J27" s="106">
         <v>1</v>
       </c>
-      <c r="K27" s="5">
+      <c r="K27" s="107">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="L27" s="33" t="s">
-        <v>25</v>
-      </c>
-      <c r="M27" s="21">
-        <v>4.5010000000000003</v>
-      </c>
-      <c r="N27" s="22">
+      <c r="L27" s="108" t="s">
+        <v>163</v>
+      </c>
+      <c r="M27" s="109"/>
+      <c r="N27" s="110">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="O27" s="110"/>
+      <c r="P27" s="110">
         <f t="shared" si="1"/>
-        <v>4.5010000000000003</v>
-      </c>
-      <c r="O27" s="22">
-        <v>4.5010000000000003</v>
-      </c>
-      <c r="P27" s="22">
-        <f t="shared" si="2"/>
-        <v>22.505000000000003</v>
-      </c>
-      <c r="Q27" s="47"/>
+        <v>0</v>
+      </c>
+      <c r="Q27" s="126" t="s">
+        <v>164</v>
+      </c>
     </row>
     <row r="28" spans="1:17" ht="15" customHeight="1" thickBot="1">
       <c r="A28" s="3">
         <v>26</v>
       </c>
-      <c r="B28" s="82"/>
+      <c r="B28" s="100"/>
       <c r="C28" s="6" t="s">
         <v>109</v>
       </c>
-      <c r="D28" s="92" t="s">
+      <c r="D28" s="76" t="s">
         <v>110</v>
       </c>
-      <c r="E28" s="56" t="s">
+      <c r="E28" s="51" t="s">
         <v>111</v>
       </c>
-      <c r="F28" s="56" t="s">
+      <c r="F28" s="51" t="s">
         <v>112</v>
       </c>
-      <c r="G28" s="9" t="s">
+      <c r="G28" s="8" t="s">
         <v>113</v>
       </c>
-      <c r="H28" s="9" t="s">
-        <v>23</v>
-      </c>
-      <c r="I28" s="9" t="s">
-        <v>23</v>
-      </c>
-      <c r="J28" s="8">
+      <c r="H28" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="I28" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="J28" s="7">
         <v>1</v>
       </c>
-      <c r="K28" s="9">
+      <c r="K28" s="8">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="L28" s="31" t="s">
+      <c r="L28" s="30" t="s">
         <v>25</v>
       </c>
-      <c r="M28" s="24">
+      <c r="M28" s="23">
         <v>0.43</v>
       </c>
-      <c r="N28" s="25">
+      <c r="N28" s="24">
+        <f t="shared" si="2"/>
+        <v>0.43</v>
+      </c>
+      <c r="O28" s="24">
+        <v>0.43</v>
+      </c>
+      <c r="P28" s="24">
         <f t="shared" si="1"/>
-        <v>0.43</v>
-      </c>
-      <c r="O28" s="25">
-        <v>0.43</v>
-      </c>
-      <c r="P28" s="25">
-        <f t="shared" si="2"/>
         <v>2.15</v>
       </c>
-      <c r="Q28" s="48"/>
+      <c r="Q28" s="45"/>
     </row>
     <row r="29" spans="1:17" ht="15" customHeight="1" thickBot="1">
       <c r="A29" s="3">
         <v>27</v>
       </c>
-      <c r="B29" s="82"/>
+      <c r="B29" s="100"/>
       <c r="C29" s="6" t="s">
         <v>114</v>
       </c>
-      <c r="D29" s="92" t="s">
+      <c r="D29" s="76" t="s">
         <v>115</v>
       </c>
-      <c r="E29" s="56" t="s">
+      <c r="E29" s="51" t="s">
         <v>116</v>
       </c>
-      <c r="F29" s="56" t="s">
+      <c r="F29" s="51" t="s">
         <v>117</v>
       </c>
-      <c r="G29" s="9" t="s">
+      <c r="G29" s="8" t="s">
         <v>118</v>
       </c>
-      <c r="H29" s="9" t="s">
-        <v>23</v>
-      </c>
-      <c r="I29" s="9" t="s">
-        <v>23</v>
-      </c>
-      <c r="J29" s="8">
+      <c r="H29" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="I29" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="J29" s="7">
         <v>1</v>
       </c>
-      <c r="K29" s="9">
+      <c r="K29" s="8">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="L29" s="31" t="s">
+      <c r="L29" s="30" t="s">
         <v>25</v>
       </c>
-      <c r="M29" s="24">
+      <c r="M29" s="23">
         <v>1.1100000000000001</v>
       </c>
-      <c r="N29" s="25">
+      <c r="N29" s="24">
+        <f t="shared" si="2"/>
+        <v>1.1100000000000001</v>
+      </c>
+      <c r="O29" s="24">
+        <v>1.1100000000000001</v>
+      </c>
+      <c r="P29" s="24">
         <f t="shared" si="1"/>
-        <v>1.1100000000000001</v>
-      </c>
-      <c r="O29" s="25">
-        <v>1.1100000000000001</v>
-      </c>
-      <c r="P29" s="25">
-        <f t="shared" si="2"/>
         <v>5.5500000000000007</v>
       </c>
-      <c r="Q29" s="49"/>
+      <c r="Q29" s="46"/>
     </row>
     <row r="30" spans="1:17" ht="15" customHeight="1" thickBot="1">
       <c r="A30" s="3">
         <v>28</v>
       </c>
-      <c r="B30" s="83"/>
-      <c r="C30" s="66" t="s">
+      <c r="B30" s="101"/>
+      <c r="C30" s="60" t="s">
         <v>119</v>
       </c>
-      <c r="D30" s="93" t="s">
+      <c r="D30" s="77" t="s">
         <v>120</v>
       </c>
-      <c r="E30" s="12"/>
-      <c r="F30" s="57" t="s">
+      <c r="E30" s="11"/>
+      <c r="F30" s="52" t="s">
         <v>121</v>
       </c>
-      <c r="G30" s="13" t="s">
+      <c r="G30" s="12" t="s">
         <v>122</v>
       </c>
-      <c r="H30" s="13" t="s">
-        <v>23</v>
-      </c>
-      <c r="I30" s="13" t="s">
-        <v>23</v>
-      </c>
-      <c r="J30" s="12">
+      <c r="H30" s="12" t="s">
+        <v>23</v>
+      </c>
+      <c r="I30" s="12" t="s">
+        <v>23</v>
+      </c>
+      <c r="J30" s="11">
         <v>1</v>
       </c>
-      <c r="K30" s="13">
+      <c r="K30" s="12">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="L30" s="26" t="s">
-        <v>25</v>
-      </c>
-      <c r="M30" s="27">
-        <v>3.1053000000000002</v>
-      </c>
-      <c r="N30" s="28">
+      <c r="L30" s="111" t="s">
+        <v>165</v>
+      </c>
+      <c r="M30" s="26">
+        <v>1.88</v>
+      </c>
+      <c r="N30" s="27">
+        <f t="shared" si="2"/>
+        <v>1.88</v>
+      </c>
+      <c r="O30" s="27">
+        <v>1.88</v>
+      </c>
+      <c r="P30" s="27">
         <f t="shared" si="1"/>
-        <v>3.1053000000000002</v>
-      </c>
-      <c r="O30" s="28">
-        <v>3.1053000000000002</v>
-      </c>
-      <c r="P30" s="28">
-        <f t="shared" si="2"/>
-        <v>15.5265</v>
-      </c>
-      <c r="Q30" s="50"/>
+        <v>9.3999999999999986</v>
+      </c>
+      <c r="Q30" s="47"/>
     </row>
     <row r="31" spans="1:17" ht="15" customHeight="1" thickBot="1">
       <c r="A31" s="3">
         <v>29</v>
       </c>
-      <c r="B31" s="90" t="s">
+      <c r="B31" s="102" t="s">
         <v>123</v>
       </c>
-      <c r="C31" s="86" t="s">
+      <c r="C31" s="72" t="s">
         <v>124</v>
       </c>
-      <c r="D31" s="74" t="s">
+      <c r="D31" s="66" t="s">
         <v>125</v>
       </c>
-      <c r="E31" s="87" t="s">
+      <c r="E31" s="73" t="s">
         <v>59</v>
       </c>
-      <c r="F31" s="74" t="s">
+      <c r="F31" s="66" t="s">
         <v>126</v>
       </c>
-      <c r="G31" s="73" t="s">
+      <c r="G31" s="65" t="s">
         <v>127</v>
       </c>
-      <c r="H31" s="73" t="s">
-        <v>23</v>
-      </c>
-      <c r="I31" s="73" t="s">
-        <v>23</v>
-      </c>
-      <c r="J31" s="88">
+      <c r="H31" s="65" t="s">
+        <v>23</v>
+      </c>
+      <c r="I31" s="65" t="s">
+        <v>23</v>
+      </c>
+      <c r="J31" s="74">
         <v>1</v>
       </c>
-      <c r="K31" s="73">
+      <c r="K31" s="65">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="L31" s="85" t="s">
+      <c r="L31" s="71" t="s">
         <v>25</v>
       </c>
-      <c r="M31" s="75">
+      <c r="M31" s="67">
         <v>0.45</v>
       </c>
-      <c r="N31" s="76">
+      <c r="N31" s="68">
+        <f t="shared" si="2"/>
+        <v>0.45</v>
+      </c>
+      <c r="O31" s="68">
+        <v>0.45</v>
+      </c>
+      <c r="P31" s="68">
         <f t="shared" si="1"/>
-        <v>0.45</v>
-      </c>
-      <c r="O31" s="76">
-        <v>0.45</v>
-      </c>
-      <c r="P31" s="76">
-        <f t="shared" si="2"/>
         <v>2.25</v>
       </c>
-      <c r="Q31" s="89"/>
+      <c r="Q31" s="75"/>
     </row>
     <row r="32" spans="1:17" ht="16.5" thickBot="1">
       <c r="A32" s="3">
         <v>30</v>
       </c>
-      <c r="B32" s="90"/>
-      <c r="C32" s="55" t="s">
+      <c r="B32" s="102"/>
+      <c r="C32" s="112" t="s">
         <v>128</v>
       </c>
-      <c r="D32" s="67" t="s">
+      <c r="D32" s="113" t="s">
         <v>129</v>
       </c>
-      <c r="E32" s="67" t="s">
+      <c r="E32" s="113" t="s">
         <v>130</v>
       </c>
-      <c r="F32" s="67" t="s">
+      <c r="F32" s="113" t="s">
         <v>130</v>
       </c>
-      <c r="G32" s="9" t="s">
-        <v>23</v>
-      </c>
-      <c r="H32" s="9" t="s">
-        <v>23</v>
-      </c>
-      <c r="I32" s="9" t="s">
-        <v>23</v>
-      </c>
-      <c r="J32" s="7">
+      <c r="G32" s="113" t="s">
+        <v>168</v>
+      </c>
+      <c r="H32" s="113" t="s">
+        <v>168</v>
+      </c>
+      <c r="I32" s="114" t="s">
+        <v>23</v>
+      </c>
+      <c r="J32" s="115">
         <v>1</v>
       </c>
-      <c r="K32" s="9">
+      <c r="K32" s="114">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="L32" s="31" t="s">
-        <v>23</v>
-      </c>
-      <c r="M32" s="24" t="s">
-        <v>23</v>
-      </c>
-      <c r="N32" s="25" t="s">
-        <v>23</v>
-      </c>
-      <c r="O32" s="25" t="s">
-        <v>23</v>
-      </c>
-      <c r="P32" s="25" t="s">
-        <v>23</v>
-      </c>
-      <c r="Q32" s="51" t="s">
+      <c r="L32" s="122" t="s">
+        <v>166</v>
+      </c>
+      <c r="M32" s="125" t="s">
+        <v>167</v>
+      </c>
+      <c r="N32" s="125" t="s">
+        <v>168</v>
+      </c>
+      <c r="O32" s="125" t="s">
+        <v>166</v>
+      </c>
+      <c r="P32" s="125" t="s">
+        <v>166</v>
+      </c>
+      <c r="Q32" s="116" t="s">
         <v>131</v>
       </c>
     </row>
@@ -3339,86 +3444,86 @@
       <c r="A33" s="3">
         <v>31</v>
       </c>
-      <c r="B33" s="91"/>
-      <c r="C33" s="68" t="s">
+      <c r="B33" s="103"/>
+      <c r="C33" s="117" t="s">
         <v>132</v>
       </c>
-      <c r="D33" s="57" t="s">
+      <c r="D33" s="118" t="s">
         <v>133</v>
       </c>
-      <c r="E33" s="12" t="s">
+      <c r="E33" s="119" t="s">
         <v>59</v>
       </c>
-      <c r="F33" s="57" t="s">
+      <c r="F33" s="118" t="s">
         <v>134</v>
       </c>
-      <c r="G33" s="13" t="s">
-        <v>23</v>
-      </c>
-      <c r="H33" s="13" t="s">
-        <v>23</v>
-      </c>
-      <c r="I33" s="13" t="s">
-        <v>23</v>
-      </c>
-      <c r="J33" s="11">
+      <c r="G33" s="123" t="s">
+        <v>167</v>
+      </c>
+      <c r="H33" s="123" t="s">
+        <v>169</v>
+      </c>
+      <c r="I33" s="120" t="s">
+        <v>23</v>
+      </c>
+      <c r="J33" s="119">
         <v>5</v>
       </c>
-      <c r="K33" s="13">
+      <c r="K33" s="120">
         <f t="shared" si="0"/>
         <v>25</v>
       </c>
-      <c r="L33" s="36" t="s">
-        <v>23</v>
-      </c>
-      <c r="M33" s="27" t="s">
-        <v>23</v>
-      </c>
-      <c r="N33" s="28" t="s">
-        <v>23</v>
-      </c>
-      <c r="O33" s="28" t="s">
-        <v>23</v>
-      </c>
-      <c r="P33" s="28" t="s">
-        <v>23</v>
-      </c>
-      <c r="Q33" s="52" t="s">
+      <c r="L33" s="123" t="s">
+        <v>166</v>
+      </c>
+      <c r="M33" s="124" t="s">
+        <v>166</v>
+      </c>
+      <c r="N33" s="124" t="s">
+        <v>167</v>
+      </c>
+      <c r="O33" s="124" t="s">
+        <v>167</v>
+      </c>
+      <c r="P33" s="124" t="s">
+        <v>166</v>
+      </c>
+      <c r="Q33" s="121" t="s">
         <v>131</v>
       </c>
     </row>
     <row r="34" spans="1:17" ht="19.5" thickBot="1">
-      <c r="J34" s="107" t="s">
+      <c r="J34" s="97" t="s">
         <v>135</v>
       </c>
-      <c r="K34" s="107"/>
-      <c r="L34" s="107"/>
-      <c r="M34" s="107"/>
-      <c r="N34" s="37">
+      <c r="K34" s="97"/>
+      <c r="L34" s="97"/>
+      <c r="M34" s="97"/>
+      <c r="N34" s="35">
         <f>SUM(N3:N33)</f>
-        <v>19.156299999999998</v>
-      </c>
-      <c r="O34" s="38"/>
-      <c r="P34" s="37">
+        <v>13.429999999999996</v>
+      </c>
+      <c r="O34" s="36"/>
+      <c r="P34" s="35">
         <f>SUM(P3:P33)</f>
-        <v>88.961500000000001</v>
+        <v>60.330000000000005</v>
       </c>
     </row>
     <row r="35" spans="1:17" ht="18.75">
-      <c r="J35" s="108" t="s">
+      <c r="J35" s="98" t="s">
         <v>136</v>
       </c>
-      <c r="K35" s="108"/>
-      <c r="L35" s="108"/>
-      <c r="M35" s="108"/>
-      <c r="N35" s="39">
+      <c r="K35" s="98"/>
+      <c r="L35" s="98"/>
+      <c r="M35" s="98"/>
+      <c r="N35" s="37">
         <f>SUM(N3:N33)</f>
-        <v>19.156299999999998</v>
-      </c>
-      <c r="O35" s="38"/>
-      <c r="P35" s="39">
+        <v>13.429999999999996</v>
+      </c>
+      <c r="O35" s="36"/>
+      <c r="P35" s="37">
         <f>P34/5</f>
-        <v>17.792300000000001</v>
+        <v>12.066000000000001</v>
       </c>
     </row>
   </sheetData>
@@ -3434,7 +3539,7 @@
     <mergeCell ref="B7:B11"/>
   </mergeCells>
   <conditionalFormatting sqref="N32">
-    <cfRule type="dataBar" priority="4">
+    <cfRule type="dataBar" priority="5">
       <dataBar>
         <cfvo type="min"/>
         <cfvo type="max"/>
@@ -3448,7 +3553,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="P32">
-    <cfRule type="dataBar" priority="5">
+    <cfRule type="dataBar" priority="6">
       <dataBar>
         <cfvo type="min"/>
         <cfvo type="max"/>
@@ -3462,7 +3567,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="N35">
-    <cfRule type="dataBar" priority="29">
+    <cfRule type="dataBar" priority="30">
       <dataBar>
         <cfvo type="min"/>
         <cfvo type="max"/>
@@ -3476,7 +3581,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="P35">
-    <cfRule type="dataBar" priority="6">
+    <cfRule type="dataBar" priority="7">
       <dataBar>
         <cfvo type="min"/>
         <cfvo type="max"/>
@@ -3490,7 +3595,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="N15:N31 N33 N3:N13">
-    <cfRule type="dataBar" priority="8">
+    <cfRule type="dataBar" priority="9">
       <dataBar>
         <cfvo type="min"/>
         <cfvo type="max"/>
@@ -3504,7 +3609,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="P15:P31 P33 P3:P13">
-    <cfRule type="dataBar" priority="31">
+    <cfRule type="dataBar" priority="32">
       <dataBar>
         <cfvo type="min"/>
         <cfvo type="max"/>
@@ -3518,7 +3623,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Q19:Q25 Q27">
-    <cfRule type="dataBar" priority="32">
+    <cfRule type="dataBar" priority="33">
       <dataBar>
         <cfvo type="min"/>
         <cfvo type="max"/>
@@ -3532,7 +3637,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K14">
-    <cfRule type="colorScale" priority="1">
+    <cfRule type="colorScale" priority="2">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -3544,7 +3649,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="N14">
-    <cfRule type="dataBar" priority="2">
+    <cfRule type="dataBar" priority="3">
       <dataBar>
         <cfvo type="min"/>
         <cfvo type="max"/>
@@ -3558,7 +3663,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="P14">
-    <cfRule type="dataBar" priority="3">
+    <cfRule type="dataBar" priority="4">
       <dataBar>
         <cfvo type="min"/>
         <cfvo type="max"/>
@@ -3572,7 +3677,19 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K3:K13 K15:K33">
-    <cfRule type="colorScale" priority="38">
+    <cfRule type="colorScale" priority="39">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J3:J33">
+    <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -3584,37 +3701,36 @@
     </cfRule>
   </conditionalFormatting>
   <hyperlinks>
-    <hyperlink ref="L3" r:id="rId1"/>
-    <hyperlink ref="L6" r:id="rId2"/>
-    <hyperlink ref="L7" r:id="rId3"/>
-    <hyperlink ref="L12" r:id="rId4"/>
-    <hyperlink ref="L15" r:id="rId5"/>
-    <hyperlink ref="L16" r:id="rId6"/>
-    <hyperlink ref="L17" r:id="rId7"/>
-    <hyperlink ref="L18" r:id="rId8"/>
-    <hyperlink ref="L19" r:id="rId9"/>
-    <hyperlink ref="L26" r:id="rId10"/>
-    <hyperlink ref="L28" r:id="rId11"/>
-    <hyperlink ref="L29" r:id="rId12"/>
-    <hyperlink ref="L31" r:id="rId13"/>
-    <hyperlink ref="L5" r:id="rId14"/>
-    <hyperlink ref="L13" r:id="rId15"/>
-    <hyperlink ref="L20" r:id="rId16"/>
-    <hyperlink ref="L21" r:id="rId17"/>
-    <hyperlink ref="L22" r:id="rId18"/>
-    <hyperlink ref="L23" r:id="rId19"/>
-    <hyperlink ref="L24" r:id="rId20"/>
-    <hyperlink ref="L30" r:id="rId21"/>
-    <hyperlink ref="L14" r:id="rId22"/>
-    <hyperlink ref="L4" r:id="rId23"/>
-    <hyperlink ref="L8" r:id="rId24"/>
-    <hyperlink ref="L9" r:id="rId25"/>
-    <hyperlink ref="L10" r:id="rId26"/>
-    <hyperlink ref="L11" r:id="rId27"/>
-    <hyperlink ref="L27" r:id="rId28"/>
+    <hyperlink ref="L3" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
+    <hyperlink ref="L6" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
+    <hyperlink ref="L7" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
+    <hyperlink ref="L12" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
+    <hyperlink ref="L15" r:id="rId5" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
+    <hyperlink ref="L16" r:id="rId6" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
+    <hyperlink ref="L17" r:id="rId7" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
+    <hyperlink ref="L18" r:id="rId8" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
+    <hyperlink ref="L19" r:id="rId9" xr:uid="{00000000-0004-0000-0000-000008000000}"/>
+    <hyperlink ref="L26" r:id="rId10" xr:uid="{00000000-0004-0000-0000-000009000000}"/>
+    <hyperlink ref="L28" r:id="rId11" xr:uid="{00000000-0004-0000-0000-00000A000000}"/>
+    <hyperlink ref="L29" r:id="rId12" xr:uid="{00000000-0004-0000-0000-00000B000000}"/>
+    <hyperlink ref="L31" r:id="rId13" xr:uid="{00000000-0004-0000-0000-00000C000000}"/>
+    <hyperlink ref="L5" r:id="rId14" xr:uid="{00000000-0004-0000-0000-00000D000000}"/>
+    <hyperlink ref="L13" r:id="rId15" xr:uid="{00000000-0004-0000-0000-00000E000000}"/>
+    <hyperlink ref="L20" r:id="rId16" xr:uid="{00000000-0004-0000-0000-00000F000000}"/>
+    <hyperlink ref="L21" r:id="rId17" xr:uid="{00000000-0004-0000-0000-000010000000}"/>
+    <hyperlink ref="L22" r:id="rId18" xr:uid="{00000000-0004-0000-0000-000011000000}"/>
+    <hyperlink ref="L23" r:id="rId19" xr:uid="{00000000-0004-0000-0000-000012000000}"/>
+    <hyperlink ref="L24" r:id="rId20" xr:uid="{00000000-0004-0000-0000-000013000000}"/>
+    <hyperlink ref="L14" r:id="rId21" xr:uid="{00000000-0004-0000-0000-000015000000}"/>
+    <hyperlink ref="L4" r:id="rId22" xr:uid="{00000000-0004-0000-0000-000016000000}"/>
+    <hyperlink ref="L8" r:id="rId23" xr:uid="{00000000-0004-0000-0000-000017000000}"/>
+    <hyperlink ref="L9" r:id="rId24" xr:uid="{00000000-0004-0000-0000-000018000000}"/>
+    <hyperlink ref="L10" r:id="rId25" xr:uid="{00000000-0004-0000-0000-000019000000}"/>
+    <hyperlink ref="L11" r:id="rId26" xr:uid="{00000000-0004-0000-0000-00001A000000}"/>
+    <hyperlink ref="L30" r:id="rId27" xr:uid="{05BF240F-850B-4BC9-9583-123F6D7CB72F}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId29"/>
+  <pageSetup orientation="portrait" r:id="rId28"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>

</xml_diff>

<commit_message>
Digikey BOM update kr dia ha LCSC BOM remaining ha
</commit_message>
<xml_diff>
--- a/Hardware-Designing/Deliverables/BOM/Digikey BOM.xlsx
+++ b/Hardware-Designing/Deliverables/BOM/Digikey BOM.xlsx
@@ -1,21 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="24430"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="5" rupBuild="14420"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark\ShockSensor-George\Hardware-Designing\Deliverables\BOM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Github\ShockSensor-George\Hardware-Designing\Deliverables\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3EA5DE71-C923-4243-ADE7-8D9F39A7B8AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="162913"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -29,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="283" uniqueCount="170">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="287" uniqueCount="171">
   <si>
     <t>Bill of Material (BOM) for  George (Rack Monitor)</t>
   </si>
@@ -360,9 +359,6 @@
     <t>IC</t>
   </si>
   <si>
-    <t>RX TXRX MOD WIFI TRACE ANT SMD</t>
-  </si>
-  <si>
     <t>U1</t>
   </si>
   <si>
@@ -506,9 +502,6 @@
     <t>R12, R13, R14, R27</t>
   </si>
   <si>
-    <t>ESP32-WROOM-32E(4MB)</t>
-  </si>
-  <si>
     <t xml:space="preserve">MOSFET N/P-CH 60V/50V SC70-6
 </t>
   </si>
@@ -540,9 +533,6 @@
 </t>
   </si>
   <si>
-    <t>Local supplier</t>
-  </si>
-  <si>
     <t>will be arrange from custom supplier</t>
   </si>
   <si>
@@ -559,12 +549,25 @@
   </si>
   <si>
     <t>-----------</t>
+  </si>
+  <si>
+    <t>ESP32-S2-WROOM-I(4M)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">18x31x3.3mm WiFi Modules ROHS
+</t>
+  </si>
+  <si>
+    <t>----</t>
+  </si>
+  <si>
+    <t>Custom supplier</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <numFmts count="2">
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00000"/>
     <numFmt numFmtId="165" formatCode="_-[$$-409]* #,##0.00_ ;_-[$$-409]* \-#,##0.00\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
@@ -729,7 +732,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="32">
+  <borders count="31">
     <border>
       <left/>
       <right/>
@@ -1028,17 +1031,6 @@
       <bottom style="medium">
         <color auto="1"/>
       </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="medium">
-        <color auto="1"/>
-      </right>
-      <top/>
-      <bottom/>
       <diagonal/>
     </border>
     <border>
@@ -1182,12 +1174,6 @@
     <xf numFmtId="0" fontId="5" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1221,16 +1207,10 @@
     <xf numFmtId="164" fontId="4" fillId="3" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="3" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="3" borderId="7" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="3" borderId="10" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="16" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="3" borderId="18" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
@@ -1262,10 +1242,7 @@
     <xf numFmtId="164" fontId="4" fillId="3" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="3" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
     <xf numFmtId="165" fontId="10" fillId="3" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
@@ -1292,12 +1269,6 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="15" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="16" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="16" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1322,91 +1293,160 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="26" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="25" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="3" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="164" fontId="5" fillId="3" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="3" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="26" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="25" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="28" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="10" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="13" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="7" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="18" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="25" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="28" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="7" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="29" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="27" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="27" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="10" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="13" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="7" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="18" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="26" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="29" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="7" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="30" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="28" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="28" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="28" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="3" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="27" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="3" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="16" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="28" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="27" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="12" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="7" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="18" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="4" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="4" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="13" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="9" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="10" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="4" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="12" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="13" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="4" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="4" borderId="10" xfId="1" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="13" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="4" borderId="13" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="4" borderId="10" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="17" fillId="4" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="6" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1437,73 +1477,25 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="6" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="15" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="7" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="16" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="18" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="4" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="4" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="13" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="4" borderId="9" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="4" borderId="10" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="4" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="4" borderId="12" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="4" borderId="13" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="4" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="4" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="4" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="4" borderId="10" xfId="1" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="4" borderId="13" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="14" fillId="4" borderId="13" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="14" fillId="4" borderId="10" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="17" fillId="4" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="16" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="16" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="4" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1781,7 +1773,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:Q35"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
@@ -1796,7 +1788,7 @@
     <col min="9" max="9" width="6.42578125" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="22.140625" customWidth="1"/>
     <col min="11" max="11" width="11.42578125" customWidth="1"/>
-    <col min="12" max="12" width="13.7109375" customWidth="1"/>
+    <col min="12" max="12" width="14" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="12.42578125" customWidth="1"/>
     <col min="14" max="14" width="13.42578125" customWidth="1"/>
     <col min="15" max="15" width="20.5703125" customWidth="1"/>
@@ -1805,31 +1797,31 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="16.5" thickBot="1">
-      <c r="A1" s="94" t="s">
+      <c r="A1" s="110" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="95"/>
-      <c r="C1" s="95"/>
-      <c r="D1" s="95"/>
-      <c r="E1" s="95"/>
-      <c r="F1" s="95"/>
-      <c r="G1" s="95"/>
-      <c r="H1" s="95"/>
-      <c r="I1" s="95"/>
-      <c r="J1" s="95"/>
-      <c r="K1" s="95"/>
-      <c r="L1" s="95"/>
-      <c r="M1" s="95"/>
-      <c r="N1" s="95"/>
-      <c r="O1" s="95"/>
-      <c r="P1" s="95"/>
-      <c r="Q1" s="96"/>
+      <c r="B1" s="111"/>
+      <c r="C1" s="111"/>
+      <c r="D1" s="111"/>
+      <c r="E1" s="111"/>
+      <c r="F1" s="111"/>
+      <c r="G1" s="111"/>
+      <c r="H1" s="111"/>
+      <c r="I1" s="111"/>
+      <c r="J1" s="111"/>
+      <c r="K1" s="111"/>
+      <c r="L1" s="111"/>
+      <c r="M1" s="111"/>
+      <c r="N1" s="111"/>
+      <c r="O1" s="111"/>
+      <c r="P1" s="111"/>
+      <c r="Q1" s="112"/>
     </row>
     <row r="2" spans="1:17" ht="16.5" thickBot="1">
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="61" t="s">
+      <c r="B2" s="54" t="s">
         <v>2</v>
       </c>
       <c r="C2" s="2" t="s">
@@ -1859,7 +1851,7 @@
       <c r="K2" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="L2" s="62" t="s">
+      <c r="L2" s="55" t="s">
         <v>12</v>
       </c>
       <c r="M2" s="2" t="s">
@@ -1871,7 +1863,7 @@
       <c r="O2" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="P2" s="63" t="s">
+      <c r="P2" s="56" t="s">
         <v>16</v>
       </c>
       <c r="Q2" s="2" t="s">
@@ -1882,81 +1874,81 @@
       <c r="A3" s="3">
         <v>1</v>
       </c>
-      <c r="B3" s="99" t="s">
+      <c r="B3" s="115" t="s">
         <v>18</v>
       </c>
       <c r="C3" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="D3" s="91" t="s">
-        <v>137</v>
-      </c>
-      <c r="E3" s="48" t="s">
+      <c r="D3" s="84" t="s">
+        <v>136</v>
+      </c>
+      <c r="E3" s="43" t="s">
         <v>20</v>
       </c>
-      <c r="F3" s="48" t="s">
+      <c r="F3" s="43" t="s">
         <v>21</v>
       </c>
-      <c r="G3" s="70" t="s">
+      <c r="G3" s="63" t="s">
         <v>22</v>
       </c>
       <c r="H3" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="I3" s="49" t="s">
+      <c r="I3" s="44" t="s">
         <v>24</v>
       </c>
-      <c r="J3" s="70">
+      <c r="J3" s="63">
         <v>6</v>
       </c>
-      <c r="K3" s="70">
+      <c r="K3" s="63">
         <f t="shared" ref="K3:K33" si="0">J3*5</f>
         <v>30</v>
       </c>
-      <c r="L3" s="92" t="s">
+      <c r="L3" s="85" t="s">
         <v>25</v>
       </c>
-      <c r="M3" s="88">
+      <c r="M3" s="81">
         <v>0.1</v>
       </c>
-      <c r="N3" s="89">
+      <c r="N3" s="82">
         <f>M3*J3</f>
         <v>0.60000000000000009</v>
       </c>
-      <c r="O3" s="88">
+      <c r="O3" s="81">
         <v>3.1E-2</v>
       </c>
-      <c r="P3" s="89">
+      <c r="P3" s="82">
         <f t="shared" ref="P3:P31" si="1">O3*K3</f>
         <v>0.92999999999999994</v>
       </c>
-      <c r="Q3" s="38"/>
+      <c r="Q3" s="34"/>
     </row>
     <row r="4" spans="1:17" ht="15.75" thickBot="1">
       <c r="A4" s="3">
         <v>2</v>
       </c>
-      <c r="B4" s="100"/>
-      <c r="C4" s="50" t="s">
+      <c r="B4" s="116"/>
+      <c r="C4" s="45" t="s">
+        <v>137</v>
+      </c>
+      <c r="D4" s="69" t="s">
         <v>138</v>
       </c>
-      <c r="D4" s="76" t="s">
+      <c r="E4" s="46" t="s">
+        <v>20</v>
+      </c>
+      <c r="F4" s="48" t="s">
         <v>139</v>
-      </c>
-      <c r="E4" s="51" t="s">
-        <v>20</v>
-      </c>
-      <c r="F4" s="53" t="s">
-        <v>140</v>
       </c>
       <c r="G4" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="H4" s="65" t="s">
-        <v>23</v>
-      </c>
-      <c r="I4" s="66" t="s">
-        <v>141</v>
+      <c r="H4" s="58" t="s">
+        <v>23</v>
+      </c>
+      <c r="I4" s="59" t="s">
+        <v>140</v>
       </c>
       <c r="J4" s="8">
         <v>1</v>
@@ -1965,40 +1957,40 @@
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="L4" s="30" t="s">
+      <c r="L4" s="27" t="s">
         <v>25</v>
       </c>
-      <c r="M4" s="23">
+      <c r="M4" s="21">
         <v>0.67</v>
       </c>
-      <c r="N4" s="24">
-        <f t="shared" ref="N3:N31" si="2">M4*J4</f>
+      <c r="N4" s="22">
+        <f t="shared" ref="N4:N31" si="2">M4*J4</f>
         <v>0.67</v>
       </c>
-      <c r="O4" s="23">
+      <c r="O4" s="21">
         <v>0.67</v>
       </c>
-      <c r="P4" s="24">
+      <c r="P4" s="22">
         <f t="shared" si="1"/>
         <v>3.35</v>
       </c>
-      <c r="Q4" s="69"/>
+      <c r="Q4" s="62"/>
     </row>
     <row r="5" spans="1:17" ht="15" customHeight="1" thickBot="1">
       <c r="A5" s="3">
         <v>3</v>
       </c>
-      <c r="B5" s="100"/>
-      <c r="C5" s="50" t="s">
+      <c r="B5" s="116"/>
+      <c r="C5" s="45" t="s">
         <v>26</v>
       </c>
-      <c r="D5" s="76" t="s">
+      <c r="D5" s="69" t="s">
         <v>27</v>
       </c>
-      <c r="E5" s="51" t="s">
+      <c r="E5" s="46" t="s">
         <v>20</v>
       </c>
-      <c r="F5" s="51" t="s">
+      <c r="F5" s="46" t="s">
         <v>28</v>
       </c>
       <c r="G5" s="8" t="s">
@@ -2017,40 +2009,40 @@
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="L5" s="22" t="s">
+      <c r="L5" s="20" t="s">
         <v>25</v>
       </c>
-      <c r="M5" s="23">
+      <c r="M5" s="21">
         <v>0.37</v>
       </c>
-      <c r="N5" s="24">
+      <c r="N5" s="22">
         <f t="shared" si="2"/>
         <v>0.74</v>
       </c>
-      <c r="O5" s="23">
+      <c r="O5" s="21">
         <v>0.25800000000000001</v>
       </c>
-      <c r="P5" s="24">
+      <c r="P5" s="22">
         <f t="shared" si="1"/>
         <v>2.58</v>
       </c>
-      <c r="Q5" s="39"/>
+      <c r="Q5" s="35"/>
     </row>
     <row r="6" spans="1:17" ht="15" customHeight="1" thickBot="1">
       <c r="A6" s="3">
         <v>4</v>
       </c>
-      <c r="B6" s="101"/>
+      <c r="B6" s="117"/>
       <c r="C6" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="D6" s="77" t="s">
+      <c r="D6" s="70" t="s">
         <v>32</v>
       </c>
-      <c r="E6" s="52" t="s">
+      <c r="E6" s="47" t="s">
         <v>20</v>
       </c>
-      <c r="F6" s="52" t="s">
+      <c r="F6" s="47" t="s">
         <v>33</v>
       </c>
       <c r="G6" s="12" t="s">
@@ -2059,7 +2051,7 @@
       <c r="H6" s="12" t="s">
         <v>23</v>
       </c>
-      <c r="I6" s="52" t="s">
+      <c r="I6" s="47" t="s">
         <v>34</v>
       </c>
       <c r="J6" s="12">
@@ -2069,98 +2061,98 @@
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="L6" s="25" t="s">
+      <c r="L6" s="23" t="s">
         <v>25</v>
       </c>
-      <c r="M6" s="26">
+      <c r="M6" s="24">
         <v>0.1</v>
       </c>
-      <c r="N6" s="27">
+      <c r="N6" s="25">
         <f t="shared" si="2"/>
         <v>0.2</v>
       </c>
-      <c r="O6" s="26">
+      <c r="O6" s="24">
         <v>3.5000000000000003E-2</v>
       </c>
-      <c r="P6" s="27">
+      <c r="P6" s="25">
         <f t="shared" si="1"/>
         <v>0.35000000000000003</v>
       </c>
-      <c r="Q6" s="40"/>
+      <c r="Q6" s="36"/>
     </row>
     <row r="7" spans="1:17" ht="16.5" customHeight="1" thickBot="1">
       <c r="A7" s="3">
         <v>5</v>
       </c>
-      <c r="B7" s="99" t="s">
+      <c r="B7" s="115" t="s">
         <v>35</v>
       </c>
-      <c r="C7" s="84" t="s">
+      <c r="C7" s="77" t="s">
         <v>36</v>
       </c>
-      <c r="D7" s="85" t="s">
-        <v>158</v>
-      </c>
-      <c r="E7" s="86" t="s">
+      <c r="D7" s="78" t="s">
+        <v>156</v>
+      </c>
+      <c r="E7" s="79" t="s">
         <v>37</v>
       </c>
-      <c r="F7" s="86" t="s">
+      <c r="F7" s="79" t="s">
         <v>38</v>
       </c>
-      <c r="G7" s="70" t="s">
+      <c r="G7" s="63" t="s">
         <v>39</v>
       </c>
-      <c r="H7" s="70" t="s">
-        <v>23</v>
-      </c>
-      <c r="I7" s="70" t="s">
-        <v>23</v>
-      </c>
-      <c r="J7" s="70">
+      <c r="H7" s="63" t="s">
+        <v>23</v>
+      </c>
+      <c r="I7" s="63" t="s">
+        <v>23</v>
+      </c>
+      <c r="J7" s="63">
         <v>1</v>
       </c>
-      <c r="K7" s="70">
+      <c r="K7" s="63">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="L7" s="87" t="s">
+      <c r="L7" s="80" t="s">
         <v>25</v>
       </c>
-      <c r="M7" s="88">
+      <c r="M7" s="81">
         <v>0.37</v>
       </c>
-      <c r="N7" s="89">
+      <c r="N7" s="82">
         <f t="shared" si="2"/>
         <v>0.37</v>
       </c>
-      <c r="O7" s="88">
+      <c r="O7" s="81">
         <v>0.37</v>
       </c>
-      <c r="P7" s="89">
+      <c r="P7" s="82">
         <f t="shared" si="1"/>
         <v>1.85</v>
       </c>
-      <c r="Q7" s="90"/>
+      <c r="Q7" s="83"/>
     </row>
     <row r="8" spans="1:17" ht="16.5" customHeight="1" thickBot="1">
       <c r="A8" s="3">
         <v>6</v>
       </c>
-      <c r="B8" s="100"/>
-      <c r="C8" s="50" t="s">
-        <v>151</v>
-      </c>
-      <c r="D8" s="76" t="s">
+      <c r="B8" s="116"/>
+      <c r="C8" s="45" t="s">
+        <v>150</v>
+      </c>
+      <c r="D8" s="69" t="s">
+        <v>141</v>
+      </c>
+      <c r="E8" s="46" t="s">
         <v>142</v>
       </c>
-      <c r="E8" s="51" t="s">
+      <c r="F8" s="46" t="s">
         <v>143</v>
       </c>
-      <c r="F8" s="51" t="s">
-        <v>144</v>
-      </c>
       <c r="G8" s="8" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="H8" s="8" t="s">
         <v>23</v>
@@ -2175,96 +2167,96 @@
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="L8" s="30" t="s">
+      <c r="L8" s="27" t="s">
         <v>25</v>
       </c>
-      <c r="M8" s="23">
+      <c r="M8" s="21">
         <v>0.39</v>
       </c>
-      <c r="N8" s="24">
+      <c r="N8" s="22">
         <f t="shared" si="2"/>
         <v>0.39</v>
       </c>
-      <c r="O8" s="23">
+      <c r="O8" s="21">
         <v>0.39</v>
       </c>
-      <c r="P8" s="24">
+      <c r="P8" s="22">
         <f t="shared" si="1"/>
         <v>1.9500000000000002</v>
       </c>
-      <c r="Q8" s="39"/>
+      <c r="Q8" s="35"/>
     </row>
     <row r="9" spans="1:17" ht="16.5" customHeight="1" thickBot="1">
       <c r="A9" s="3">
         <v>7</v>
       </c>
-      <c r="B9" s="100"/>
-      <c r="C9" s="81" t="s">
-        <v>160</v>
-      </c>
-      <c r="D9" s="80" t="s">
+      <c r="B9" s="116"/>
+      <c r="C9" s="74" t="s">
+        <v>158</v>
+      </c>
+      <c r="D9" s="73" t="s">
+        <v>144</v>
+      </c>
+      <c r="E9" s="59" t="s">
+        <v>142</v>
+      </c>
+      <c r="F9" s="50" t="s">
         <v>145</v>
       </c>
-      <c r="E9" s="66" t="s">
-        <v>143</v>
-      </c>
-      <c r="F9" s="57" t="s">
-        <v>146</v>
-      </c>
       <c r="G9" s="8" t="s">
-        <v>159</v>
-      </c>
-      <c r="H9" s="65" t="s">
-        <v>23</v>
-      </c>
-      <c r="I9" s="65" t="s">
-        <v>23</v>
-      </c>
-      <c r="J9" s="65">
+        <v>157</v>
+      </c>
+      <c r="H9" s="58" t="s">
+        <v>23</v>
+      </c>
+      <c r="I9" s="58" t="s">
+        <v>23</v>
+      </c>
+      <c r="J9" s="58">
         <v>1</v>
       </c>
       <c r="K9" s="8">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="L9" s="30" t="s">
+      <c r="L9" s="27" t="s">
         <v>25</v>
       </c>
-      <c r="M9" s="23">
+      <c r="M9" s="21">
         <v>0.52</v>
       </c>
-      <c r="N9" s="24">
+      <c r="N9" s="22">
         <f t="shared" si="2"/>
         <v>0.52</v>
       </c>
-      <c r="O9" s="23">
+      <c r="O9" s="21">
         <v>0.52</v>
       </c>
-      <c r="P9" s="24">
+      <c r="P9" s="22">
         <f t="shared" si="1"/>
         <v>2.6</v>
       </c>
-      <c r="Q9" s="39"/>
+      <c r="Q9" s="35"/>
     </row>
     <row r="10" spans="1:17" ht="16.5" customHeight="1" thickBot="1">
       <c r="A10" s="3">
         <v>8</v>
       </c>
-      <c r="B10" s="100"/>
-      <c r="C10" s="50" t="s">
-        <v>161</v>
-      </c>
-      <c r="D10" s="76" t="s">
+      <c r="B10" s="116"/>
+      <c r="C10" s="45" t="s">
+        <v>159</v>
+      </c>
+      <c r="D10" s="69" t="s">
+        <v>146</v>
+      </c>
+      <c r="E10" s="46" t="s">
+        <v>142</v>
+      </c>
+      <c r="F10" s="48" t="s">
         <v>147</v>
       </c>
-      <c r="E10" s="51" t="s">
-        <v>143</v>
-      </c>
-      <c r="F10" s="53" t="s">
-        <v>148</v>
-      </c>
       <c r="G10" s="8" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="H10" s="8" t="s">
         <v>23</v>
@@ -2279,44 +2271,44 @@
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="L10" s="30" t="s">
+      <c r="L10" s="27" t="s">
         <v>25</v>
       </c>
-      <c r="M10" s="23">
+      <c r="M10" s="21">
         <v>0.25</v>
       </c>
-      <c r="N10" s="24">
+      <c r="N10" s="22">
         <f t="shared" si="2"/>
         <v>0.25</v>
       </c>
-      <c r="O10" s="23">
+      <c r="O10" s="21">
         <v>0.25</v>
       </c>
-      <c r="P10" s="24">
+      <c r="P10" s="22">
         <f t="shared" si="1"/>
         <v>1.25</v>
       </c>
-      <c r="Q10" s="39"/>
+      <c r="Q10" s="35"/>
     </row>
     <row r="11" spans="1:17" ht="16.5" customHeight="1" thickBot="1">
       <c r="A11" s="3">
         <v>9</v>
       </c>
-      <c r="B11" s="101"/>
-      <c r="C11" s="93" t="s">
-        <v>162</v>
-      </c>
-      <c r="D11" s="77" t="s">
+      <c r="B11" s="117"/>
+      <c r="C11" s="86" t="s">
+        <v>160</v>
+      </c>
+      <c r="D11" s="70" t="s">
+        <v>148</v>
+      </c>
+      <c r="E11" s="47" t="s">
+        <v>142</v>
+      </c>
+      <c r="F11" s="47" t="s">
         <v>149</v>
       </c>
-      <c r="E11" s="52" t="s">
-        <v>143</v>
-      </c>
-      <c r="F11" s="52" t="s">
-        <v>150</v>
-      </c>
       <c r="G11" s="12" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="H11" s="12" t="s">
         <v>23</v>
@@ -2331,42 +2323,42 @@
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="L11" s="25" t="s">
+      <c r="L11" s="23" t="s">
         <v>25</v>
       </c>
-      <c r="M11" s="26">
+      <c r="M11" s="24">
         <v>0.37</v>
       </c>
-      <c r="N11" s="27">
+      <c r="N11" s="25">
         <f t="shared" si="2"/>
         <v>0.37</v>
       </c>
-      <c r="O11" s="26">
+      <c r="O11" s="24">
         <v>0.37</v>
       </c>
-      <c r="P11" s="27">
+      <c r="P11" s="25">
         <f t="shared" si="1"/>
         <v>1.85</v>
       </c>
-      <c r="Q11" s="40"/>
+      <c r="Q11" s="36"/>
     </row>
     <row r="12" spans="1:17" ht="15.75" thickBot="1">
       <c r="A12" s="3">
         <v>10</v>
       </c>
-      <c r="B12" s="99" t="s">
+      <c r="B12" s="115" t="s">
         <v>40</v>
       </c>
-      <c r="C12" s="82" t="s">
+      <c r="C12" s="75" t="s">
         <v>41</v>
       </c>
-      <c r="D12" s="83" t="s">
+      <c r="D12" s="76" t="s">
         <v>42</v>
       </c>
-      <c r="E12" s="48" t="s">
+      <c r="E12" s="43" t="s">
         <v>43</v>
       </c>
-      <c r="F12" s="48" t="s">
+      <c r="F12" s="43" t="s">
         <v>44</v>
       </c>
       <c r="G12" s="5" t="s">
@@ -2385,40 +2377,40 @@
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="L12" s="29" t="s">
+      <c r="L12" s="26" t="s">
         <v>25</v>
       </c>
-      <c r="M12" s="20">
+      <c r="M12" s="18">
         <v>0.44</v>
       </c>
-      <c r="N12" s="21">
+      <c r="N12" s="19">
         <f t="shared" si="2"/>
         <v>0.44</v>
       </c>
-      <c r="O12" s="20">
+      <c r="O12" s="18">
         <v>0.44</v>
       </c>
-      <c r="P12" s="21">
+      <c r="P12" s="19">
         <f t="shared" si="1"/>
         <v>2.2000000000000002</v>
       </c>
-      <c r="Q12" s="38"/>
+      <c r="Q12" s="34"/>
     </row>
     <row r="13" spans="1:17" ht="15" customHeight="1" thickBot="1">
       <c r="A13" s="3">
         <v>11</v>
       </c>
-      <c r="B13" s="100"/>
+      <c r="B13" s="116"/>
       <c r="C13" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="D13" s="76" t="s">
+      <c r="D13" s="69" t="s">
         <v>47</v>
       </c>
-      <c r="E13" s="51" t="s">
+      <c r="E13" s="46" t="s">
         <v>48</v>
       </c>
-      <c r="F13" s="51" t="s">
+      <c r="F13" s="46" t="s">
         <v>49</v>
       </c>
       <c r="G13" s="8" t="s">
@@ -2437,41 +2429,41 @@
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="L13" s="30" t="s">
+      <c r="L13" s="27" t="s">
         <v>25</v>
       </c>
-      <c r="M13" s="23">
+      <c r="M13" s="21">
         <v>0.14000000000000001</v>
       </c>
-      <c r="N13" s="24">
+      <c r="N13" s="22">
         <f t="shared" si="2"/>
         <v>0.28000000000000003</v>
       </c>
-      <c r="O13" s="23">
+      <c r="O13" s="21">
         <v>0.13200000000000001</v>
       </c>
-      <c r="P13" s="24">
+      <c r="P13" s="22">
         <f t="shared" si="1"/>
         <v>1.32</v>
       </c>
-      <c r="Q13" s="39"/>
+      <c r="Q13" s="35"/>
     </row>
     <row r="14" spans="1:17" ht="15" customHeight="1" thickBot="1">
       <c r="A14" s="3">
         <v>12</v>
       </c>
-      <c r="B14" s="101"/>
+      <c r="B14" s="117"/>
       <c r="C14" s="9" t="s">
+        <v>152</v>
+      </c>
+      <c r="D14" s="10" t="s">
+        <v>153</v>
+      </c>
+      <c r="E14" s="47" t="s">
         <v>154</v>
       </c>
-      <c r="D14" s="10" t="s">
+      <c r="F14" s="47" t="s">
         <v>155</v>
-      </c>
-      <c r="E14" s="52" t="s">
-        <v>156</v>
-      </c>
-      <c r="F14" s="52" t="s">
-        <v>157</v>
       </c>
       <c r="G14" s="12" t="s">
         <v>45</v>
@@ -2489,42 +2481,42 @@
         <f>J14*5</f>
         <v>5</v>
       </c>
-      <c r="L14" s="25" t="s">
+      <c r="L14" s="23" t="s">
         <v>25</v>
       </c>
-      <c r="M14" s="26">
+      <c r="M14" s="24">
         <v>0.55000000000000004</v>
       </c>
-      <c r="N14" s="27">
+      <c r="N14" s="25">
         <f>M14*J14</f>
         <v>0.55000000000000004</v>
       </c>
-      <c r="O14" s="26">
+      <c r="O14" s="24">
         <v>0.55000000000000004</v>
       </c>
-      <c r="P14" s="27">
+      <c r="P14" s="25">
         <f>O14*K14</f>
         <v>2.75</v>
       </c>
-      <c r="Q14" s="40"/>
+      <c r="Q14" s="36"/>
     </row>
     <row r="15" spans="1:17" ht="16.5" customHeight="1" thickBot="1">
       <c r="A15" s="3">
         <v>13</v>
       </c>
-      <c r="B15" s="99" t="s">
+      <c r="B15" s="115" t="s">
         <v>50</v>
       </c>
       <c r="C15" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="D15" s="78" t="s">
+      <c r="D15" s="71" t="s">
         <v>52</v>
       </c>
-      <c r="E15" s="49" t="s">
+      <c r="E15" s="44" t="s">
         <v>53</v>
       </c>
-      <c r="F15" s="49" t="s">
+      <c r="F15" s="44" t="s">
         <v>54</v>
       </c>
       <c r="G15" s="5" t="s">
@@ -2533,7 +2525,7 @@
       <c r="H15" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="I15" s="49" t="s">
+      <c r="I15" s="44" t="s">
         <v>56</v>
       </c>
       <c r="J15" s="13">
@@ -2543,40 +2535,40 @@
         <f t="shared" si="0"/>
         <v>25</v>
       </c>
-      <c r="L15" s="29" t="s">
+      <c r="L15" s="26" t="s">
         <v>25</v>
       </c>
-      <c r="M15" s="20">
+      <c r="M15" s="18">
         <v>0.1</v>
       </c>
-      <c r="N15" s="21">
+      <c r="N15" s="19">
         <f t="shared" si="2"/>
         <v>0.5</v>
       </c>
-      <c r="O15" s="20">
+      <c r="O15" s="18">
         <v>5.8000000000000003E-2</v>
       </c>
-      <c r="P15" s="21">
+      <c r="P15" s="19">
         <f t="shared" si="1"/>
         <v>1.4500000000000002</v>
       </c>
-      <c r="Q15" s="38"/>
+      <c r="Q15" s="34"/>
     </row>
     <row r="16" spans="1:17" ht="15" customHeight="1" thickBot="1">
       <c r="A16" s="3">
         <v>14</v>
       </c>
-      <c r="B16" s="100"/>
-      <c r="C16" s="54" t="s">
+      <c r="B16" s="116"/>
+      <c r="C16" s="49" t="s">
         <v>57</v>
       </c>
-      <c r="D16" s="76" t="s">
+      <c r="D16" s="69" t="s">
         <v>58</v>
       </c>
       <c r="E16" s="7" t="s">
         <v>59</v>
       </c>
-      <c r="F16" s="51" t="s">
+      <c r="F16" s="46" t="s">
         <v>60</v>
       </c>
       <c r="G16" s="8" t="s">
@@ -2585,7 +2577,7 @@
       <c r="H16" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="I16" s="51" t="s">
+      <c r="I16" s="46" t="s">
         <v>56</v>
       </c>
       <c r="J16" s="7">
@@ -2595,40 +2587,40 @@
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="L16" s="30" t="s">
+      <c r="L16" s="27" t="s">
         <v>25</v>
       </c>
-      <c r="M16" s="23">
+      <c r="M16" s="21">
         <v>0.26</v>
       </c>
-      <c r="N16" s="24">
+      <c r="N16" s="22">
         <f t="shared" si="2"/>
         <v>0.26</v>
       </c>
-      <c r="O16" s="23">
+      <c r="O16" s="21">
         <v>0.26</v>
       </c>
-      <c r="P16" s="24">
+      <c r="P16" s="22">
         <f t="shared" si="1"/>
         <v>1.3</v>
       </c>
-      <c r="Q16" s="39"/>
+      <c r="Q16" s="35"/>
     </row>
     <row r="17" spans="1:17" ht="15" customHeight="1" thickBot="1">
       <c r="A17" s="3">
         <v>15</v>
       </c>
-      <c r="B17" s="100"/>
-      <c r="C17" s="54" t="s">
+      <c r="B17" s="116"/>
+      <c r="C17" s="49" t="s">
         <v>62</v>
       </c>
-      <c r="D17" s="76" t="s">
+      <c r="D17" s="69" t="s">
         <v>63</v>
       </c>
-      <c r="E17" s="51" t="s">
+      <c r="E17" s="46" t="s">
         <v>53</v>
       </c>
-      <c r="F17" s="51" t="s">
+      <c r="F17" s="46" t="s">
         <v>64</v>
       </c>
       <c r="G17" s="8" t="s">
@@ -2637,7 +2629,7 @@
       <c r="H17" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="I17" s="51" t="s">
+      <c r="I17" s="46" t="s">
         <v>66</v>
       </c>
       <c r="J17" s="7">
@@ -2647,40 +2639,40 @@
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="L17" s="30" t="s">
+      <c r="L17" s="27" t="s">
         <v>25</v>
       </c>
-      <c r="M17" s="23">
+      <c r="M17" s="21">
         <v>0.1</v>
       </c>
-      <c r="N17" s="24">
+      <c r="N17" s="22">
         <f t="shared" si="2"/>
         <v>0.2</v>
       </c>
-      <c r="O17" s="23">
+      <c r="O17" s="21">
         <v>0.1</v>
       </c>
-      <c r="P17" s="24">
+      <c r="P17" s="22">
         <f t="shared" si="1"/>
         <v>1</v>
       </c>
-      <c r="Q17" s="39"/>
+      <c r="Q17" s="35"/>
     </row>
     <row r="18" spans="1:17" ht="15" customHeight="1" thickBot="1">
       <c r="A18" s="3">
         <v>16</v>
       </c>
-      <c r="B18" s="100"/>
+      <c r="B18" s="116"/>
       <c r="C18" s="6" t="s">
         <v>67</v>
       </c>
-      <c r="D18" s="76" t="s">
+      <c r="D18" s="69" t="s">
         <v>68</v>
       </c>
-      <c r="E18" s="51" t="s">
+      <c r="E18" s="46" t="s">
         <v>53</v>
       </c>
-      <c r="F18" s="51" t="s">
+      <c r="F18" s="46" t="s">
         <v>69</v>
       </c>
       <c r="G18" s="8" t="s">
@@ -2689,7 +2681,7 @@
       <c r="H18" s="14" t="s">
         <v>23</v>
       </c>
-      <c r="I18" s="51" t="s">
+      <c r="I18" s="46" t="s">
         <v>70</v>
       </c>
       <c r="J18" s="7">
@@ -2699,40 +2691,40 @@
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="L18" s="30" t="s">
+      <c r="L18" s="27" t="s">
         <v>25</v>
       </c>
-      <c r="M18" s="23">
+      <c r="M18" s="21">
         <v>0.1</v>
       </c>
-      <c r="N18" s="24">
+      <c r="N18" s="22">
         <f t="shared" si="2"/>
         <v>0.1</v>
       </c>
-      <c r="O18" s="23">
+      <c r="O18" s="21">
         <v>0.1</v>
       </c>
-      <c r="P18" s="24">
+      <c r="P18" s="22">
         <f t="shared" si="1"/>
         <v>0.5</v>
       </c>
-      <c r="Q18" s="39"/>
+      <c r="Q18" s="35"/>
     </row>
     <row r="19" spans="1:17" ht="15" customHeight="1" thickBot="1">
       <c r="A19" s="3">
         <v>17</v>
       </c>
-      <c r="B19" s="100"/>
+      <c r="B19" s="116"/>
       <c r="C19" s="6" t="s">
         <v>71</v>
       </c>
-      <c r="D19" s="76" t="s">
-        <v>152</v>
-      </c>
-      <c r="E19" s="51" t="s">
+      <c r="D19" s="69" t="s">
+        <v>151</v>
+      </c>
+      <c r="E19" s="46" t="s">
         <v>53</v>
       </c>
-      <c r="F19" s="51" t="s">
+      <c r="F19" s="46" t="s">
         <v>72</v>
       </c>
       <c r="G19" s="8" t="s">
@@ -2741,7 +2733,7 @@
       <c r="H19" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="I19" s="51" t="s">
+      <c r="I19" s="46" t="s">
         <v>73</v>
       </c>
       <c r="J19" s="7">
@@ -2751,40 +2743,40 @@
         <f t="shared" si="0"/>
         <v>20</v>
       </c>
-      <c r="L19" s="30" t="s">
+      <c r="L19" s="27" t="s">
         <v>25</v>
       </c>
-      <c r="M19" s="24">
+      <c r="M19" s="22">
         <v>0.1</v>
       </c>
-      <c r="N19" s="24">
+      <c r="N19" s="22">
         <f t="shared" si="2"/>
         <v>0.4</v>
       </c>
-      <c r="O19" s="24">
+      <c r="O19" s="22">
         <v>2.4E-2</v>
       </c>
-      <c r="P19" s="24">
+      <c r="P19" s="22">
         <f t="shared" si="1"/>
         <v>0.48</v>
       </c>
-      <c r="Q19" s="41"/>
+      <c r="Q19" s="37"/>
     </row>
     <row r="20" spans="1:17" ht="15" customHeight="1" thickBot="1">
       <c r="A20" s="3">
         <v>18</v>
       </c>
-      <c r="B20" s="100"/>
-      <c r="C20" s="54" t="s">
+      <c r="B20" s="116"/>
+      <c r="C20" s="49" t="s">
         <v>74</v>
       </c>
-      <c r="D20" s="76" t="s">
+      <c r="D20" s="69" t="s">
         <v>75</v>
       </c>
-      <c r="E20" s="51" t="s">
+      <c r="E20" s="46" t="s">
         <v>53</v>
       </c>
-      <c r="F20" s="51" t="s">
+      <c r="F20" s="46" t="s">
         <v>76</v>
       </c>
       <c r="G20" s="8" t="s">
@@ -2803,40 +2795,40 @@
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="L20" s="30" t="s">
+      <c r="L20" s="27" t="s">
         <v>25</v>
       </c>
-      <c r="M20" s="24">
+      <c r="M20" s="22">
         <v>0.1</v>
       </c>
-      <c r="N20" s="24">
+      <c r="N20" s="22">
         <f t="shared" si="2"/>
         <v>0.1</v>
       </c>
-      <c r="O20" s="24">
+      <c r="O20" s="22">
         <v>0.1</v>
       </c>
-      <c r="P20" s="24">
+      <c r="P20" s="22">
         <f t="shared" si="1"/>
         <v>0.5</v>
       </c>
-      <c r="Q20" s="41"/>
+      <c r="Q20" s="37"/>
     </row>
     <row r="21" spans="1:17" ht="15" customHeight="1" thickBot="1">
       <c r="A21" s="3">
         <v>19</v>
       </c>
-      <c r="B21" s="100"/>
-      <c r="C21" s="54" t="s">
+      <c r="B21" s="116"/>
+      <c r="C21" s="49" t="s">
         <v>79</v>
       </c>
-      <c r="D21" s="76" t="s">
+      <c r="D21" s="69" t="s">
         <v>80</v>
       </c>
-      <c r="E21" s="51" t="s">
+      <c r="E21" s="46" t="s">
         <v>53</v>
       </c>
-      <c r="F21" s="51" t="s">
+      <c r="F21" s="46" t="s">
         <v>81</v>
       </c>
       <c r="G21" s="8" t="s">
@@ -2855,40 +2847,40 @@
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="L21" s="30" t="s">
+      <c r="L21" s="27" t="s">
         <v>25</v>
       </c>
-      <c r="M21" s="24">
+      <c r="M21" s="22">
         <v>0.1</v>
       </c>
-      <c r="N21" s="24">
+      <c r="N21" s="22">
         <f t="shared" si="2"/>
         <v>0.1</v>
       </c>
-      <c r="O21" s="24">
+      <c r="O21" s="22">
         <v>0.1</v>
       </c>
-      <c r="P21" s="24">
+      <c r="P21" s="22">
         <f t="shared" si="1"/>
         <v>0.5</v>
       </c>
-      <c r="Q21" s="41"/>
+      <c r="Q21" s="37"/>
     </row>
     <row r="22" spans="1:17" ht="15" customHeight="1" thickBot="1">
       <c r="A22" s="3">
         <v>20</v>
       </c>
-      <c r="B22" s="100"/>
+      <c r="B22" s="116"/>
       <c r="C22" s="6" t="s">
         <v>84</v>
       </c>
-      <c r="D22" s="76" t="s">
+      <c r="D22" s="69" t="s">
         <v>85</v>
       </c>
-      <c r="E22" s="51" t="s">
+      <c r="E22" s="46" t="s">
         <v>53</v>
       </c>
-      <c r="F22" s="51" t="s">
+      <c r="F22" s="46" t="s">
         <v>86</v>
       </c>
       <c r="G22" s="8" t="s">
@@ -2907,40 +2899,40 @@
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="L22" s="30" t="s">
+      <c r="L22" s="27" t="s">
         <v>25</v>
       </c>
-      <c r="M22" s="24">
+      <c r="M22" s="22">
         <v>0.1</v>
       </c>
-      <c r="N22" s="24">
+      <c r="N22" s="22">
         <f t="shared" si="2"/>
         <v>0.1</v>
       </c>
-      <c r="O22" s="24">
+      <c r="O22" s="22">
         <v>0.1</v>
       </c>
-      <c r="P22" s="24">
+      <c r="P22" s="22">
         <f t="shared" si="1"/>
         <v>0.5</v>
       </c>
-      <c r="Q22" s="41"/>
+      <c r="Q22" s="37"/>
     </row>
     <row r="23" spans="1:17" ht="15" customHeight="1" thickBot="1">
       <c r="A23" s="3">
         <v>21</v>
       </c>
-      <c r="B23" s="100"/>
-      <c r="C23" s="54" t="s">
+      <c r="B23" s="116"/>
+      <c r="C23" s="49" t="s">
         <v>88</v>
       </c>
-      <c r="D23" s="76" t="s">
+      <c r="D23" s="69" t="s">
         <v>89</v>
       </c>
-      <c r="E23" s="51" t="s">
+      <c r="E23" s="46" t="s">
         <v>53</v>
       </c>
-      <c r="F23" s="51" t="s">
+      <c r="F23" s="46" t="s">
         <v>90</v>
       </c>
       <c r="G23" s="8" t="s">
@@ -2959,40 +2951,40 @@
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="L23" s="30" t="s">
+      <c r="L23" s="27" t="s">
         <v>25</v>
       </c>
-      <c r="M23" s="24">
+      <c r="M23" s="22">
         <v>0.1</v>
       </c>
-      <c r="N23" s="24">
+      <c r="N23" s="22">
         <f t="shared" si="2"/>
         <v>0.1</v>
       </c>
-      <c r="O23" s="24">
+      <c r="O23" s="22">
         <v>0.1</v>
       </c>
-      <c r="P23" s="24">
+      <c r="P23" s="22">
         <f t="shared" si="1"/>
         <v>0.5</v>
       </c>
-      <c r="Q23" s="41"/>
+      <c r="Q23" s="37"/>
     </row>
     <row r="24" spans="1:17" ht="15.75" thickBot="1">
       <c r="A24" s="3">
         <v>22</v>
       </c>
-      <c r="B24" s="101"/>
+      <c r="B24" s="117"/>
       <c r="C24" s="9" t="s">
         <v>92</v>
       </c>
-      <c r="D24" s="77" t="s">
+      <c r="D24" s="70" t="s">
         <v>93</v>
       </c>
-      <c r="E24" s="52" t="s">
+      <c r="E24" s="47" t="s">
         <v>53</v>
       </c>
-      <c r="F24" s="52" t="s">
+      <c r="F24" s="47" t="s">
         <v>94</v>
       </c>
       <c r="G24" s="12" t="s">
@@ -3011,194 +3003,210 @@
         <f t="shared" si="0"/>
         <v>20</v>
       </c>
-      <c r="L24" s="25" t="s">
+      <c r="L24" s="23" t="s">
         <v>25</v>
       </c>
-      <c r="M24" s="27">
+      <c r="M24" s="25">
         <v>0.1</v>
       </c>
-      <c r="N24" s="27">
+      <c r="N24" s="25">
         <f t="shared" si="2"/>
         <v>0.4</v>
       </c>
-      <c r="O24" s="27">
+      <c r="O24" s="25">
         <v>0.1</v>
       </c>
-      <c r="P24" s="27">
+      <c r="P24" s="25">
         <f t="shared" si="1"/>
         <v>2</v>
       </c>
-      <c r="Q24" s="42"/>
+      <c r="Q24" s="38"/>
     </row>
     <row r="25" spans="1:17" ht="16.5" thickBot="1">
       <c r="A25" s="3">
         <v>23</v>
       </c>
-      <c r="B25" s="64" t="s">
+      <c r="B25" s="57" t="s">
         <v>96</v>
       </c>
-      <c r="C25" s="55" t="s">
+      <c r="C25" s="120" t="s">
         <v>97</v>
       </c>
-      <c r="D25" s="56" t="s">
+      <c r="D25" s="121" t="s">
         <v>98</v>
       </c>
-      <c r="E25" s="15" t="s">
+      <c r="E25" s="122" t="s">
         <v>59</v>
       </c>
-      <c r="F25" s="57" t="s">
+      <c r="F25" s="121" t="s">
         <v>99</v>
       </c>
-      <c r="G25" s="16"/>
-      <c r="H25" s="16"/>
-      <c r="I25" s="16" t="s">
-        <v>23</v>
-      </c>
-      <c r="J25" s="16">
+      <c r="G25" s="123" t="s">
+        <v>163</v>
+      </c>
+      <c r="H25" s="123" t="s">
+        <v>169</v>
+      </c>
+      <c r="I25" s="124" t="s">
+        <v>23</v>
+      </c>
+      <c r="J25" s="124">
         <v>1</v>
       </c>
-      <c r="K25" s="16">
+      <c r="K25" s="124">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="L25" s="31"/>
-      <c r="M25" s="28"/>
-      <c r="N25" s="28">
+      <c r="L25" s="125" t="s">
+        <v>170</v>
+      </c>
+      <c r="M25" s="126">
+        <v>1.2</v>
+      </c>
+      <c r="N25" s="126">
         <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="O25" s="28"/>
-      <c r="P25" s="28">
+        <v>1.2</v>
+      </c>
+      <c r="O25" s="126">
+        <v>1.2</v>
+      </c>
+      <c r="P25" s="126">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="Q25" s="43"/>
+        <v>6</v>
+      </c>
+      <c r="Q25" s="108" t="s">
+        <v>161</v>
+      </c>
     </row>
     <row r="26" spans="1:17" ht="16.5" thickBot="1">
       <c r="A26" s="3">
         <v>24</v>
       </c>
-      <c r="B26" s="17" t="s">
+      <c r="B26" s="15" t="s">
         <v>100</v>
       </c>
-      <c r="C26" s="58" t="s">
+      <c r="C26" s="51" t="s">
         <v>101</v>
       </c>
-      <c r="D26" s="79" t="s">
+      <c r="D26" s="72" t="s">
         <v>102</v>
       </c>
-      <c r="E26" s="18" t="s">
+      <c r="E26" s="16" t="s">
         <v>59</v>
       </c>
-      <c r="F26" s="59" t="s">
+      <c r="F26" s="52" t="s">
         <v>103</v>
       </c>
-      <c r="G26" s="19" t="s">
+      <c r="G26" s="17" t="s">
         <v>104</v>
       </c>
-      <c r="H26" s="19" t="s">
-        <v>23</v>
-      </c>
-      <c r="I26" s="19" t="s">
-        <v>23</v>
-      </c>
-      <c r="J26" s="19">
+      <c r="H26" s="17" t="s">
+        <v>23</v>
+      </c>
+      <c r="I26" s="17" t="s">
+        <v>23</v>
+      </c>
+      <c r="J26" s="17">
         <v>2</v>
       </c>
-      <c r="K26" s="19">
+      <c r="K26" s="17">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="L26" s="32" t="s">
+      <c r="L26" s="28" t="s">
         <v>25</v>
       </c>
-      <c r="M26" s="33">
+      <c r="M26" s="29">
         <v>0.96</v>
       </c>
-      <c r="N26" s="34">
+      <c r="N26" s="30">
         <f t="shared" si="2"/>
         <v>1.92</v>
       </c>
-      <c r="O26" s="34">
+      <c r="O26" s="30">
         <v>0.92700000000000005</v>
       </c>
-      <c r="P26" s="34">
+      <c r="P26" s="30">
         <f t="shared" si="1"/>
         <v>9.27</v>
       </c>
-      <c r="Q26" s="44"/>
+      <c r="Q26" s="39"/>
     </row>
     <row r="27" spans="1:17" ht="15" customHeight="1" thickBot="1">
       <c r="A27" s="3">
         <v>25</v>
       </c>
-      <c r="B27" s="99" t="s">
+      <c r="B27" s="115" t="s">
         <v>105</v>
       </c>
-      <c r="C27" s="104" t="s">
+      <c r="C27" s="109" t="s">
+        <v>168</v>
+      </c>
+      <c r="D27" s="87" t="s">
         <v>106</v>
       </c>
-      <c r="D27" s="105" t="s">
+      <c r="E27" s="88" t="s">
+        <v>59</v>
+      </c>
+      <c r="F27" s="88" t="s">
+        <v>167</v>
+      </c>
+      <c r="G27" s="89" t="s">
         <v>107</v>
       </c>
-      <c r="E27" s="106" t="s">
-        <v>59</v>
-      </c>
-      <c r="F27" s="105" t="s">
-        <v>153</v>
-      </c>
-      <c r="G27" s="107" t="s">
-        <v>108</v>
-      </c>
-      <c r="H27" s="107" t="s">
-        <v>23</v>
-      </c>
-      <c r="I27" s="107" t="s">
-        <v>23</v>
-      </c>
-      <c r="J27" s="106">
+      <c r="H27" s="89" t="s">
+        <v>23</v>
+      </c>
+      <c r="I27" s="89" t="s">
+        <v>23</v>
+      </c>
+      <c r="J27" s="88">
         <v>1</v>
       </c>
-      <c r="K27" s="107">
+      <c r="K27" s="89">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="L27" s="108" t="s">
-        <v>163</v>
-      </c>
-      <c r="M27" s="109"/>
-      <c r="N27" s="110">
+      <c r="L27" s="90" t="s">
+        <v>170</v>
+      </c>
+      <c r="M27" s="91">
+        <v>4.8</v>
+      </c>
+      <c r="N27" s="92">
         <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="O27" s="110"/>
-      <c r="P27" s="110">
+        <v>4.8</v>
+      </c>
+      <c r="O27" s="92">
+        <v>4.8</v>
+      </c>
+      <c r="P27" s="92">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="Q27" s="126" t="s">
-        <v>164</v>
+        <v>24</v>
+      </c>
+      <c r="Q27" s="108" t="s">
+        <v>161</v>
       </c>
     </row>
     <row r="28" spans="1:17" ht="15" customHeight="1" thickBot="1">
       <c r="A28" s="3">
         <v>26</v>
       </c>
-      <c r="B28" s="100"/>
+      <c r="B28" s="116"/>
       <c r="C28" s="6" t="s">
+        <v>108</v>
+      </c>
+      <c r="D28" s="69" t="s">
         <v>109</v>
       </c>
-      <c r="D28" s="76" t="s">
+      <c r="E28" s="46" t="s">
         <v>110</v>
       </c>
-      <c r="E28" s="51" t="s">
+      <c r="F28" s="46" t="s">
         <v>111</v>
       </c>
-      <c r="F28" s="51" t="s">
+      <c r="G28" s="8" t="s">
         <v>112</v>
-      </c>
-      <c r="G28" s="8" t="s">
-        <v>113</v>
       </c>
       <c r="H28" s="8" t="s">
         <v>23</v>
@@ -3213,44 +3221,44 @@
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="L28" s="30" t="s">
+      <c r="L28" s="27" t="s">
         <v>25</v>
       </c>
-      <c r="M28" s="23">
+      <c r="M28" s="21">
         <v>0.43</v>
       </c>
-      <c r="N28" s="24">
+      <c r="N28" s="22">
         <f t="shared" si="2"/>
         <v>0.43</v>
       </c>
-      <c r="O28" s="24">
+      <c r="O28" s="22">
         <v>0.43</v>
       </c>
-      <c r="P28" s="24">
+      <c r="P28" s="22">
         <f t="shared" si="1"/>
         <v>2.15</v>
       </c>
-      <c r="Q28" s="45"/>
+      <c r="Q28" s="40"/>
     </row>
     <row r="29" spans="1:17" ht="15" customHeight="1" thickBot="1">
       <c r="A29" s="3">
         <v>27</v>
       </c>
-      <c r="B29" s="100"/>
+      <c r="B29" s="116"/>
       <c r="C29" s="6" t="s">
+        <v>113</v>
+      </c>
+      <c r="D29" s="69" t="s">
         <v>114</v>
       </c>
-      <c r="D29" s="76" t="s">
+      <c r="E29" s="46" t="s">
         <v>115</v>
       </c>
-      <c r="E29" s="51" t="s">
+      <c r="F29" s="46" t="s">
         <v>116</v>
       </c>
-      <c r="F29" s="51" t="s">
+      <c r="G29" s="8" t="s">
         <v>117</v>
-      </c>
-      <c r="G29" s="8" t="s">
-        <v>118</v>
       </c>
       <c r="H29" s="8" t="s">
         <v>23</v>
@@ -3265,42 +3273,42 @@
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="L29" s="30" t="s">
+      <c r="L29" s="27" t="s">
         <v>25</v>
       </c>
-      <c r="M29" s="23">
+      <c r="M29" s="21">
         <v>1.1100000000000001</v>
       </c>
-      <c r="N29" s="24">
+      <c r="N29" s="22">
         <f t="shared" si="2"/>
         <v>1.1100000000000001</v>
       </c>
-      <c r="O29" s="24">
+      <c r="O29" s="22">
         <v>1.1100000000000001</v>
       </c>
-      <c r="P29" s="24">
+      <c r="P29" s="22">
         <f t="shared" si="1"/>
         <v>5.5500000000000007</v>
       </c>
-      <c r="Q29" s="46"/>
+      <c r="Q29" s="41"/>
     </row>
     <row r="30" spans="1:17" ht="15" customHeight="1" thickBot="1">
       <c r="A30" s="3">
         <v>28</v>
       </c>
-      <c r="B30" s="101"/>
-      <c r="C30" s="60" t="s">
+      <c r="B30" s="117"/>
+      <c r="C30" s="53" t="s">
+        <v>118</v>
+      </c>
+      <c r="D30" s="70" t="s">
         <v>119</v>
       </c>
-      <c r="D30" s="77" t="s">
+      <c r="E30" s="11"/>
+      <c r="F30" s="47" t="s">
         <v>120</v>
       </c>
-      <c r="E30" s="11"/>
-      <c r="F30" s="52" t="s">
+      <c r="G30" s="12" t="s">
         <v>121</v>
-      </c>
-      <c r="G30" s="12" t="s">
-        <v>122</v>
       </c>
       <c r="H30" s="12" t="s">
         <v>23</v>
@@ -3315,215 +3323,215 @@
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="L30" s="111" t="s">
-        <v>165</v>
-      </c>
-      <c r="M30" s="26">
+      <c r="L30" s="93" t="s">
+        <v>162</v>
+      </c>
+      <c r="M30" s="24">
         <v>1.88</v>
       </c>
-      <c r="N30" s="27">
+      <c r="N30" s="25">
         <f t="shared" si="2"/>
         <v>1.88</v>
       </c>
-      <c r="O30" s="27">
+      <c r="O30" s="25">
         <v>1.88</v>
       </c>
-      <c r="P30" s="27">
+      <c r="P30" s="25">
         <f t="shared" si="1"/>
         <v>9.3999999999999986</v>
       </c>
-      <c r="Q30" s="47"/>
+      <c r="Q30" s="42"/>
     </row>
     <row r="31" spans="1:17" ht="15" customHeight="1" thickBot="1">
       <c r="A31" s="3">
         <v>29</v>
       </c>
-      <c r="B31" s="102" t="s">
+      <c r="B31" s="118" t="s">
+        <v>122</v>
+      </c>
+      <c r="C31" s="65" t="s">
         <v>123</v>
       </c>
-      <c r="C31" s="72" t="s">
+      <c r="D31" s="59" t="s">
         <v>124</v>
       </c>
-      <c r="D31" s="66" t="s">
+      <c r="E31" s="66" t="s">
+        <v>59</v>
+      </c>
+      <c r="F31" s="59" t="s">
         <v>125</v>
       </c>
-      <c r="E31" s="73" t="s">
-        <v>59</v>
-      </c>
-      <c r="F31" s="66" t="s">
+      <c r="G31" s="58" t="s">
         <v>126</v>
       </c>
-      <c r="G31" s="65" t="s">
-        <v>127</v>
-      </c>
-      <c r="H31" s="65" t="s">
-        <v>23</v>
-      </c>
-      <c r="I31" s="65" t="s">
-        <v>23</v>
-      </c>
-      <c r="J31" s="74">
+      <c r="H31" s="58" t="s">
+        <v>23</v>
+      </c>
+      <c r="I31" s="58" t="s">
+        <v>23</v>
+      </c>
+      <c r="J31" s="67">
         <v>1</v>
       </c>
-      <c r="K31" s="65">
+      <c r="K31" s="58">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="L31" s="71" t="s">
+      <c r="L31" s="64" t="s">
         <v>25</v>
       </c>
-      <c r="M31" s="67">
+      <c r="M31" s="60">
         <v>0.45</v>
       </c>
-      <c r="N31" s="68">
+      <c r="N31" s="61">
         <f t="shared" si="2"/>
         <v>0.45</v>
       </c>
-      <c r="O31" s="68">
+      <c r="O31" s="61">
         <v>0.45</v>
       </c>
-      <c r="P31" s="68">
+      <c r="P31" s="61">
         <f t="shared" si="1"/>
         <v>2.25</v>
       </c>
-      <c r="Q31" s="75"/>
+      <c r="Q31" s="68"/>
     </row>
     <row r="32" spans="1:17" ht="16.5" thickBot="1">
       <c r="A32" s="3">
         <v>30</v>
       </c>
-      <c r="B32" s="102"/>
-      <c r="C32" s="112" t="s">
+      <c r="B32" s="118"/>
+      <c r="C32" s="94" t="s">
+        <v>127</v>
+      </c>
+      <c r="D32" s="95" t="s">
         <v>128</v>
       </c>
-      <c r="D32" s="113" t="s">
+      <c r="E32" s="95" t="s">
         <v>129</v>
       </c>
-      <c r="E32" s="113" t="s">
-        <v>130</v>
-      </c>
-      <c r="F32" s="113" t="s">
-        <v>130</v>
-      </c>
-      <c r="G32" s="113" t="s">
-        <v>168</v>
-      </c>
-      <c r="H32" s="113" t="s">
-        <v>168</v>
-      </c>
-      <c r="I32" s="114" t="s">
-        <v>23</v>
-      </c>
-      <c r="J32" s="115">
+      <c r="F32" s="95" t="s">
+        <v>129</v>
+      </c>
+      <c r="G32" s="95" t="s">
+        <v>165</v>
+      </c>
+      <c r="H32" s="95" t="s">
+        <v>165</v>
+      </c>
+      <c r="I32" s="96" t="s">
+        <v>23</v>
+      </c>
+      <c r="J32" s="97">
         <v>1</v>
       </c>
-      <c r="K32" s="114">
+      <c r="K32" s="96">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="L32" s="122" t="s">
-        <v>166</v>
-      </c>
-      <c r="M32" s="125" t="s">
-        <v>167</v>
-      </c>
-      <c r="N32" s="125" t="s">
-        <v>168</v>
-      </c>
-      <c r="O32" s="125" t="s">
-        <v>166</v>
-      </c>
-      <c r="P32" s="125" t="s">
-        <v>166</v>
-      </c>
-      <c r="Q32" s="116" t="s">
-        <v>131</v>
+      <c r="L32" s="104" t="s">
+        <v>163</v>
+      </c>
+      <c r="M32" s="107" t="s">
+        <v>164</v>
+      </c>
+      <c r="N32" s="107" t="s">
+        <v>165</v>
+      </c>
+      <c r="O32" s="107" t="s">
+        <v>163</v>
+      </c>
+      <c r="P32" s="107" t="s">
+        <v>163</v>
+      </c>
+      <c r="Q32" s="98" t="s">
+        <v>130</v>
       </c>
     </row>
     <row r="33" spans="1:17" ht="16.5" thickBot="1">
       <c r="A33" s="3">
         <v>31</v>
       </c>
-      <c r="B33" s="103"/>
-      <c r="C33" s="117" t="s">
+      <c r="B33" s="119"/>
+      <c r="C33" s="99" t="s">
+        <v>131</v>
+      </c>
+      <c r="D33" s="100" t="s">
         <v>132</v>
       </c>
-      <c r="D33" s="118" t="s">
+      <c r="E33" s="101" t="s">
+        <v>59</v>
+      </c>
+      <c r="F33" s="100" t="s">
         <v>133</v>
       </c>
-      <c r="E33" s="119" t="s">
-        <v>59</v>
-      </c>
-      <c r="F33" s="118" t="s">
-        <v>134</v>
-      </c>
-      <c r="G33" s="123" t="s">
-        <v>167</v>
-      </c>
-      <c r="H33" s="123" t="s">
-        <v>169</v>
-      </c>
-      <c r="I33" s="120" t="s">
-        <v>23</v>
-      </c>
-      <c r="J33" s="119">
+      <c r="G33" s="105" t="s">
+        <v>164</v>
+      </c>
+      <c r="H33" s="105" t="s">
+        <v>166</v>
+      </c>
+      <c r="I33" s="102" t="s">
+        <v>23</v>
+      </c>
+      <c r="J33" s="101">
         <v>5</v>
       </c>
-      <c r="K33" s="120">
+      <c r="K33" s="102">
         <f t="shared" si="0"/>
         <v>25</v>
       </c>
-      <c r="L33" s="123" t="s">
-        <v>166</v>
-      </c>
-      <c r="M33" s="124" t="s">
-        <v>166</v>
-      </c>
-      <c r="N33" s="124" t="s">
-        <v>167</v>
-      </c>
-      <c r="O33" s="124" t="s">
-        <v>167</v>
-      </c>
-      <c r="P33" s="124" t="s">
-        <v>166</v>
-      </c>
-      <c r="Q33" s="121" t="s">
-        <v>131</v>
+      <c r="L33" s="105" t="s">
+        <v>163</v>
+      </c>
+      <c r="M33" s="106" t="s">
+        <v>163</v>
+      </c>
+      <c r="N33" s="106" t="s">
+        <v>164</v>
+      </c>
+      <c r="O33" s="106" t="s">
+        <v>164</v>
+      </c>
+      <c r="P33" s="106" t="s">
+        <v>163</v>
+      </c>
+      <c r="Q33" s="103" t="s">
+        <v>130</v>
       </c>
     </row>
     <row r="34" spans="1:17" ht="19.5" thickBot="1">
-      <c r="J34" s="97" t="s">
-        <v>135</v>
-      </c>
-      <c r="K34" s="97"/>
-      <c r="L34" s="97"/>
-      <c r="M34" s="97"/>
-      <c r="N34" s="35">
+      <c r="J34" s="113" t="s">
+        <v>134</v>
+      </c>
+      <c r="K34" s="113"/>
+      <c r="L34" s="113"/>
+      <c r="M34" s="113"/>
+      <c r="N34" s="31">
         <f>SUM(N3:N33)</f>
-        <v>13.429999999999996</v>
-      </c>
-      <c r="O34" s="36"/>
-      <c r="P34" s="35">
+        <v>19.429999999999996</v>
+      </c>
+      <c r="O34" s="32"/>
+      <c r="P34" s="31">
         <f>SUM(P3:P33)</f>
-        <v>60.330000000000005</v>
+        <v>90.330000000000013</v>
       </c>
     </row>
     <row r="35" spans="1:17" ht="18.75">
-      <c r="J35" s="98" t="s">
-        <v>136</v>
-      </c>
-      <c r="K35" s="98"/>
-      <c r="L35" s="98"/>
-      <c r="M35" s="98"/>
-      <c r="N35" s="37">
+      <c r="J35" s="114" t="s">
+        <v>135</v>
+      </c>
+      <c r="K35" s="114"/>
+      <c r="L35" s="114"/>
+      <c r="M35" s="114"/>
+      <c r="N35" s="33">
         <f>SUM(N3:N33)</f>
-        <v>13.429999999999996</v>
-      </c>
-      <c r="O35" s="36"/>
-      <c r="P35" s="37">
+        <v>19.429999999999996</v>
+      </c>
+      <c r="O35" s="32"/>
+      <c r="P35" s="33">
         <f>P34/5</f>
-        <v>12.066000000000001</v>
+        <v>18.066000000000003</v>
       </c>
     </row>
   </sheetData>
@@ -3701,33 +3709,33 @@
     </cfRule>
   </conditionalFormatting>
   <hyperlinks>
-    <hyperlink ref="L3" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
-    <hyperlink ref="L6" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
-    <hyperlink ref="L7" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
-    <hyperlink ref="L12" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
-    <hyperlink ref="L15" r:id="rId5" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
-    <hyperlink ref="L16" r:id="rId6" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
-    <hyperlink ref="L17" r:id="rId7" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
-    <hyperlink ref="L18" r:id="rId8" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
-    <hyperlink ref="L19" r:id="rId9" xr:uid="{00000000-0004-0000-0000-000008000000}"/>
-    <hyperlink ref="L26" r:id="rId10" xr:uid="{00000000-0004-0000-0000-000009000000}"/>
-    <hyperlink ref="L28" r:id="rId11" xr:uid="{00000000-0004-0000-0000-00000A000000}"/>
-    <hyperlink ref="L29" r:id="rId12" xr:uid="{00000000-0004-0000-0000-00000B000000}"/>
-    <hyperlink ref="L31" r:id="rId13" xr:uid="{00000000-0004-0000-0000-00000C000000}"/>
-    <hyperlink ref="L5" r:id="rId14" xr:uid="{00000000-0004-0000-0000-00000D000000}"/>
-    <hyperlink ref="L13" r:id="rId15" xr:uid="{00000000-0004-0000-0000-00000E000000}"/>
-    <hyperlink ref="L20" r:id="rId16" xr:uid="{00000000-0004-0000-0000-00000F000000}"/>
-    <hyperlink ref="L21" r:id="rId17" xr:uid="{00000000-0004-0000-0000-000010000000}"/>
-    <hyperlink ref="L22" r:id="rId18" xr:uid="{00000000-0004-0000-0000-000011000000}"/>
-    <hyperlink ref="L23" r:id="rId19" xr:uid="{00000000-0004-0000-0000-000012000000}"/>
-    <hyperlink ref="L24" r:id="rId20" xr:uid="{00000000-0004-0000-0000-000013000000}"/>
-    <hyperlink ref="L14" r:id="rId21" xr:uid="{00000000-0004-0000-0000-000015000000}"/>
-    <hyperlink ref="L4" r:id="rId22" xr:uid="{00000000-0004-0000-0000-000016000000}"/>
-    <hyperlink ref="L8" r:id="rId23" xr:uid="{00000000-0004-0000-0000-000017000000}"/>
-    <hyperlink ref="L9" r:id="rId24" xr:uid="{00000000-0004-0000-0000-000018000000}"/>
-    <hyperlink ref="L10" r:id="rId25" xr:uid="{00000000-0004-0000-0000-000019000000}"/>
-    <hyperlink ref="L11" r:id="rId26" xr:uid="{00000000-0004-0000-0000-00001A000000}"/>
-    <hyperlink ref="L30" r:id="rId27" xr:uid="{05BF240F-850B-4BC9-9583-123F6D7CB72F}"/>
+    <hyperlink ref="L3" r:id="rId1"/>
+    <hyperlink ref="L6" r:id="rId2"/>
+    <hyperlink ref="L7" r:id="rId3"/>
+    <hyperlink ref="L12" r:id="rId4"/>
+    <hyperlink ref="L15" r:id="rId5"/>
+    <hyperlink ref="L16" r:id="rId6"/>
+    <hyperlink ref="L17" r:id="rId7"/>
+    <hyperlink ref="L18" r:id="rId8"/>
+    <hyperlink ref="L19" r:id="rId9"/>
+    <hyperlink ref="L26" r:id="rId10"/>
+    <hyperlink ref="L28" r:id="rId11"/>
+    <hyperlink ref="L29" r:id="rId12"/>
+    <hyperlink ref="L31" r:id="rId13"/>
+    <hyperlink ref="L5" r:id="rId14"/>
+    <hyperlink ref="L13" r:id="rId15"/>
+    <hyperlink ref="L20" r:id="rId16"/>
+    <hyperlink ref="L21" r:id="rId17"/>
+    <hyperlink ref="L22" r:id="rId18"/>
+    <hyperlink ref="L23" r:id="rId19"/>
+    <hyperlink ref="L24" r:id="rId20"/>
+    <hyperlink ref="L14" r:id="rId21"/>
+    <hyperlink ref="L4" r:id="rId22"/>
+    <hyperlink ref="L8" r:id="rId23"/>
+    <hyperlink ref="L9" r:id="rId24"/>
+    <hyperlink ref="L10" r:id="rId25"/>
+    <hyperlink ref="L11" r:id="rId26"/>
+    <hyperlink ref="L30" r:id="rId27"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId28"/>

</xml_diff>

<commit_message>
#10 LCSC BOM Update kr dia ha jo parts LCSC per Non stock han wo Quotation k lye issue per mention kr diye han
</commit_message>
<xml_diff>
--- a/Hardware-Designing/Deliverables/BOM/Digikey BOM.xlsx
+++ b/Hardware-Designing/Deliverables/BOM/Digikey BOM.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="287" uniqueCount="171">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="288" uniqueCount="172">
   <si>
     <t>Bill of Material (BOM) for  George (Rack Monitor)</t>
   </si>
@@ -562,6 +562,9 @@
   </si>
   <si>
     <t>Custom supplier</t>
+  </si>
+  <si>
+    <t>QFN-24</t>
   </si>
 </sst>
 </file>
@@ -585,7 +588,7 @@
       <sz val="12"/>
       <color theme="0"/>
       <name val="Calibri"/>
-      <charset val="134"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -593,28 +596,28 @@
       <sz val="11"/>
       <color theme="0"/>
       <name val="Calibri"/>
-      <charset val="134"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <b/>
       <sz val="12"/>
       <name val="Calibri"/>
-      <charset val="134"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="10"/>
       <color theme="1"/>
       <name val="Calibri"/>
-      <charset val="134"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
-      <charset val="134"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -622,7 +625,7 @@
       <sz val="12"/>
       <color theme="1"/>
       <name val="Calibri"/>
-      <charset val="134"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -630,7 +633,7 @@
       <sz val="10"/>
       <color theme="10"/>
       <name val="Calibri"/>
-      <charset val="134"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -638,18 +641,18 @@
       <sz val="10"/>
       <color theme="10"/>
       <name val="Calibri"/>
-      <charset val="134"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="14"/>
       <name val="Calibri"/>
-      <charset val="134"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="10"/>
       <name val="Calibri"/>
-      <charset val="134"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -657,7 +660,7 @@
       <sz val="10"/>
       <color theme="10"/>
       <name val="Arial"/>
-      <charset val="134"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
@@ -1447,6 +1450,27 @@
     <xf numFmtId="0" fontId="4" fillId="4" borderId="6" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="15" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="16" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="16" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="16" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="4" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1475,27 +1499,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="15" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="16" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="16" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="16" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="4" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1797,25 +1800,25 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="16.5" thickBot="1">
-      <c r="A1" s="110" t="s">
+      <c r="A1" s="117" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="111"/>
-      <c r="C1" s="111"/>
-      <c r="D1" s="111"/>
-      <c r="E1" s="111"/>
-      <c r="F1" s="111"/>
-      <c r="G1" s="111"/>
-      <c r="H1" s="111"/>
-      <c r="I1" s="111"/>
-      <c r="J1" s="111"/>
-      <c r="K1" s="111"/>
-      <c r="L1" s="111"/>
-      <c r="M1" s="111"/>
-      <c r="N1" s="111"/>
-      <c r="O1" s="111"/>
-      <c r="P1" s="111"/>
-      <c r="Q1" s="112"/>
+      <c r="B1" s="118"/>
+      <c r="C1" s="118"/>
+      <c r="D1" s="118"/>
+      <c r="E1" s="118"/>
+      <c r="F1" s="118"/>
+      <c r="G1" s="118"/>
+      <c r="H1" s="118"/>
+      <c r="I1" s="118"/>
+      <c r="J1" s="118"/>
+      <c r="K1" s="118"/>
+      <c r="L1" s="118"/>
+      <c r="M1" s="118"/>
+      <c r="N1" s="118"/>
+      <c r="O1" s="118"/>
+      <c r="P1" s="118"/>
+      <c r="Q1" s="119"/>
     </row>
     <row r="2" spans="1:17" ht="16.5" thickBot="1">
       <c r="A2" s="1" t="s">
@@ -1874,7 +1877,7 @@
       <c r="A3" s="3">
         <v>1</v>
       </c>
-      <c r="B3" s="115" t="s">
+      <c r="B3" s="122" t="s">
         <v>18</v>
       </c>
       <c r="C3" s="4" t="s">
@@ -1928,7 +1931,7 @@
       <c r="A4" s="3">
         <v>2</v>
       </c>
-      <c r="B4" s="116"/>
+      <c r="B4" s="123"/>
       <c r="C4" s="45" t="s">
         <v>137</v>
       </c>
@@ -1980,7 +1983,7 @@
       <c r="A5" s="3">
         <v>3</v>
       </c>
-      <c r="B5" s="116"/>
+      <c r="B5" s="123"/>
       <c r="C5" s="45" t="s">
         <v>26</v>
       </c>
@@ -2032,7 +2035,7 @@
       <c r="A6" s="3">
         <v>4</v>
       </c>
-      <c r="B6" s="117"/>
+      <c r="B6" s="124"/>
       <c r="C6" s="9" t="s">
         <v>31</v>
       </c>
@@ -2084,7 +2087,7 @@
       <c r="A7" s="3">
         <v>5</v>
       </c>
-      <c r="B7" s="115" t="s">
+      <c r="B7" s="122" t="s">
         <v>35</v>
       </c>
       <c r="C7" s="77" t="s">
@@ -2138,7 +2141,7 @@
       <c r="A8" s="3">
         <v>6</v>
       </c>
-      <c r="B8" s="116"/>
+      <c r="B8" s="123"/>
       <c r="C8" s="45" t="s">
         <v>150</v>
       </c>
@@ -2190,7 +2193,7 @@
       <c r="A9" s="3">
         <v>7</v>
       </c>
-      <c r="B9" s="116"/>
+      <c r="B9" s="123"/>
       <c r="C9" s="74" t="s">
         <v>158</v>
       </c>
@@ -2242,7 +2245,7 @@
       <c r="A10" s="3">
         <v>8</v>
       </c>
-      <c r="B10" s="116"/>
+      <c r="B10" s="123"/>
       <c r="C10" s="45" t="s">
         <v>159</v>
       </c>
@@ -2294,7 +2297,7 @@
       <c r="A11" s="3">
         <v>9</v>
       </c>
-      <c r="B11" s="117"/>
+      <c r="B11" s="124"/>
       <c r="C11" s="86" t="s">
         <v>160</v>
       </c>
@@ -2346,7 +2349,7 @@
       <c r="A12" s="3">
         <v>10</v>
       </c>
-      <c r="B12" s="115" t="s">
+      <c r="B12" s="122" t="s">
         <v>40</v>
       </c>
       <c r="C12" s="75" t="s">
@@ -2400,7 +2403,7 @@
       <c r="A13" s="3">
         <v>11</v>
       </c>
-      <c r="B13" s="116"/>
+      <c r="B13" s="123"/>
       <c r="C13" s="6" t="s">
         <v>46</v>
       </c>
@@ -2452,7 +2455,7 @@
       <c r="A14" s="3">
         <v>12</v>
       </c>
-      <c r="B14" s="117"/>
+      <c r="B14" s="124"/>
       <c r="C14" s="9" t="s">
         <v>152</v>
       </c>
@@ -2504,7 +2507,7 @@
       <c r="A15" s="3">
         <v>13</v>
       </c>
-      <c r="B15" s="115" t="s">
+      <c r="B15" s="122" t="s">
         <v>50</v>
       </c>
       <c r="C15" s="4" t="s">
@@ -2558,7 +2561,7 @@
       <c r="A16" s="3">
         <v>14</v>
       </c>
-      <c r="B16" s="116"/>
+      <c r="B16" s="123"/>
       <c r="C16" s="49" t="s">
         <v>57</v>
       </c>
@@ -2610,7 +2613,7 @@
       <c r="A17" s="3">
         <v>15</v>
       </c>
-      <c r="B17" s="116"/>
+      <c r="B17" s="123"/>
       <c r="C17" s="49" t="s">
         <v>62</v>
       </c>
@@ -2662,7 +2665,7 @@
       <c r="A18" s="3">
         <v>16</v>
       </c>
-      <c r="B18" s="116"/>
+      <c r="B18" s="123"/>
       <c r="C18" s="6" t="s">
         <v>67</v>
       </c>
@@ -2714,7 +2717,7 @@
       <c r="A19" s="3">
         <v>17</v>
       </c>
-      <c r="B19" s="116"/>
+      <c r="B19" s="123"/>
       <c r="C19" s="6" t="s">
         <v>71</v>
       </c>
@@ -2766,7 +2769,7 @@
       <c r="A20" s="3">
         <v>18</v>
       </c>
-      <c r="B20" s="116"/>
+      <c r="B20" s="123"/>
       <c r="C20" s="49" t="s">
         <v>74</v>
       </c>
@@ -2818,7 +2821,7 @@
       <c r="A21" s="3">
         <v>19</v>
       </c>
-      <c r="B21" s="116"/>
+      <c r="B21" s="123"/>
       <c r="C21" s="49" t="s">
         <v>79</v>
       </c>
@@ -2870,7 +2873,7 @@
       <c r="A22" s="3">
         <v>20</v>
       </c>
-      <c r="B22" s="116"/>
+      <c r="B22" s="123"/>
       <c r="C22" s="6" t="s">
         <v>84</v>
       </c>
@@ -2922,7 +2925,7 @@
       <c r="A23" s="3">
         <v>21</v>
       </c>
-      <c r="B23" s="116"/>
+      <c r="B23" s="123"/>
       <c r="C23" s="49" t="s">
         <v>88</v>
       </c>
@@ -2974,7 +2977,7 @@
       <c r="A24" s="3">
         <v>22</v>
       </c>
-      <c r="B24" s="117"/>
+      <c r="B24" s="124"/>
       <c r="C24" s="9" t="s">
         <v>92</v>
       </c>
@@ -3029,48 +3032,48 @@
       <c r="B25" s="57" t="s">
         <v>96</v>
       </c>
-      <c r="C25" s="120" t="s">
+      <c r="C25" s="110" t="s">
         <v>97</v>
       </c>
-      <c r="D25" s="121" t="s">
+      <c r="D25" s="111" t="s">
         <v>98</v>
       </c>
-      <c r="E25" s="122" t="s">
+      <c r="E25" s="112" t="s">
         <v>59</v>
       </c>
-      <c r="F25" s="121" t="s">
+      <c r="F25" s="111" t="s">
         <v>99</v>
       </c>
-      <c r="G25" s="123" t="s">
+      <c r="G25" s="113" t="s">
         <v>163</v>
       </c>
-      <c r="H25" s="123" t="s">
+      <c r="H25" s="113" t="s">
         <v>169</v>
       </c>
-      <c r="I25" s="124" t="s">
-        <v>23</v>
-      </c>
-      <c r="J25" s="124">
+      <c r="I25" s="114" t="s">
+        <v>23</v>
+      </c>
+      <c r="J25" s="114">
         <v>1</v>
       </c>
-      <c r="K25" s="124">
+      <c r="K25" s="114">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="L25" s="125" t="s">
+      <c r="L25" s="115" t="s">
         <v>170</v>
       </c>
-      <c r="M25" s="126">
+      <c r="M25" s="116">
         <v>1.2</v>
       </c>
-      <c r="N25" s="126">
+      <c r="N25" s="116">
         <f t="shared" si="2"/>
         <v>1.2</v>
       </c>
-      <c r="O25" s="126">
+      <c r="O25" s="116">
         <v>1.2</v>
       </c>
-      <c r="P25" s="126">
+      <c r="P25" s="116">
         <f t="shared" si="1"/>
         <v>6</v>
       </c>
@@ -3136,7 +3139,7 @@
       <c r="A27" s="3">
         <v>25</v>
       </c>
-      <c r="B27" s="115" t="s">
+      <c r="B27" s="122" t="s">
         <v>105</v>
       </c>
       <c r="C27" s="109" t="s">
@@ -3192,7 +3195,7 @@
       <c r="A28" s="3">
         <v>26</v>
       </c>
-      <c r="B28" s="116"/>
+      <c r="B28" s="123"/>
       <c r="C28" s="6" t="s">
         <v>108</v>
       </c>
@@ -3244,7 +3247,7 @@
       <c r="A29" s="3">
         <v>27</v>
       </c>
-      <c r="B29" s="116"/>
+      <c r="B29" s="123"/>
       <c r="C29" s="6" t="s">
         <v>113</v>
       </c>
@@ -3296,14 +3299,16 @@
       <c r="A30" s="3">
         <v>28</v>
       </c>
-      <c r="B30" s="117"/>
+      <c r="B30" s="124"/>
       <c r="C30" s="53" t="s">
         <v>118</v>
       </c>
       <c r="D30" s="70" t="s">
         <v>119</v>
       </c>
-      <c r="E30" s="11"/>
+      <c r="E30" s="11" t="s">
+        <v>171</v>
+      </c>
       <c r="F30" s="47" t="s">
         <v>120</v>
       </c>
@@ -3346,7 +3351,7 @@
       <c r="A31" s="3">
         <v>29</v>
       </c>
-      <c r="B31" s="118" t="s">
+      <c r="B31" s="125" t="s">
         <v>122</v>
       </c>
       <c r="C31" s="65" t="s">
@@ -3400,7 +3405,7 @@
       <c r="A32" s="3">
         <v>30</v>
       </c>
-      <c r="B32" s="118"/>
+      <c r="B32" s="125"/>
       <c r="C32" s="94" t="s">
         <v>127</v>
       </c>
@@ -3452,7 +3457,7 @@
       <c r="A33" s="3">
         <v>31</v>
       </c>
-      <c r="B33" s="119"/>
+      <c r="B33" s="126"/>
       <c r="C33" s="99" t="s">
         <v>131</v>
       </c>
@@ -3501,12 +3506,12 @@
       </c>
     </row>
     <row r="34" spans="1:17" ht="19.5" thickBot="1">
-      <c r="J34" s="113" t="s">
+      <c r="J34" s="120" t="s">
         <v>134</v>
       </c>
-      <c r="K34" s="113"/>
-      <c r="L34" s="113"/>
-      <c r="M34" s="113"/>
+      <c r="K34" s="120"/>
+      <c r="L34" s="120"/>
+      <c r="M34" s="120"/>
       <c r="N34" s="31">
         <f>SUM(N3:N33)</f>
         <v>19.429999999999996</v>
@@ -3518,12 +3523,12 @@
       </c>
     </row>
     <row r="35" spans="1:17" ht="18.75">
-      <c r="J35" s="114" t="s">
+      <c r="J35" s="121" t="s">
         <v>135</v>
       </c>
-      <c r="K35" s="114"/>
-      <c r="L35" s="114"/>
-      <c r="M35" s="114"/>
+      <c r="K35" s="121"/>
+      <c r="L35" s="121"/>
+      <c r="M35" s="121"/>
       <c r="N35" s="33">
         <f>SUM(N3:N33)</f>
         <v>19.429999999999996</v>

</xml_diff>